<commit_message>
feature adendum fisrt commit
</commit_message>
<xml_diff>
--- a/backend/final_schedule.xlsx
+++ b/backend/final_schedule.xlsx
@@ -1605,13 +1605,13 @@
         <v>1</v>
       </c>
       <c r="I29" s="18" t="n">
-        <v>1999280.8</v>
+        <v>1999280</v>
       </c>
       <c r="J29" s="18" t="n">
-        <v>1999280.8</v>
+        <v>0</v>
       </c>
       <c r="K29" s="17" t="n">
-        <v>0.55759234</v>
+        <v>0</v>
       </c>
       <c r="L29" s="11" t="n"/>
       <c r="M29" s="20" t="n">
@@ -1724,10 +1724,10 @@
         <v>300000</v>
       </c>
       <c r="J32" s="18" t="n">
-        <v>300000</v>
+        <v>0</v>
       </c>
       <c r="K32" s="17" t="n">
-        <v>0.08366897</v>
+        <v>0</v>
       </c>
       <c r="L32" s="11" t="n"/>
       <c r="M32" s="20" t="n">
@@ -1784,10 +1784,10 @@
         <v>150000</v>
       </c>
       <c r="J33" s="18" t="n">
-        <v>150000</v>
+        <v>0</v>
       </c>
       <c r="K33" s="17" t="n">
-        <v>0.04183449</v>
+        <v>0</v>
       </c>
       <c r="L33" s="11" t="n"/>
       <c r="M33" s="20" t="n">
@@ -1900,10 +1900,10 @@
         <v>25000</v>
       </c>
       <c r="J36" s="18" t="n">
-        <v>125000</v>
+        <v>0</v>
       </c>
       <c r="K36" s="17" t="n">
-        <v>0.03486207</v>
+        <v>0</v>
       </c>
       <c r="L36" s="11" t="n"/>
       <c r="M36" s="20" t="n">
@@ -1960,10 +1960,10 @@
         <v>60000</v>
       </c>
       <c r="J37" s="18" t="n">
-        <v>60000</v>
+        <v>0</v>
       </c>
       <c r="K37" s="17" t="n">
-        <v>0.01673379</v>
+        <v>0</v>
       </c>
       <c r="L37" s="11" t="n"/>
       <c r="M37" s="20" t="n">
@@ -2020,10 +2020,10 @@
         <v>68000</v>
       </c>
       <c r="J38" s="18" t="n">
-        <v>340000</v>
+        <v>0</v>
       </c>
       <c r="K38" s="17" t="n">
-        <v>0.09482483999999999</v>
+        <v>0</v>
       </c>
       <c r="L38" s="11" t="n"/>
       <c r="M38" s="20" t="n">
@@ -2080,10 +2080,10 @@
         <v>35000</v>
       </c>
       <c r="J39" s="18" t="n">
-        <v>175000</v>
+        <v>0</v>
       </c>
       <c r="K39" s="17" t="n">
-        <v>0.0488069</v>
+        <v>0</v>
       </c>
       <c r="L39" s="11" t="n"/>
       <c r="M39" s="20" t="n">
@@ -2196,10 +2196,10 @@
         <v>800000</v>
       </c>
       <c r="J42" s="18" t="n">
-        <v>800000</v>
+        <v>0</v>
       </c>
       <c r="K42" s="17" t="n">
-        <v>0.22311726</v>
+        <v>0</v>
       </c>
       <c r="L42" s="11" t="n"/>
       <c r="M42" s="20" t="n">
@@ -2312,10 +2312,10 @@
         <v>1500000</v>
       </c>
       <c r="J45" s="18" t="n">
-        <v>1500000</v>
+        <v>0</v>
       </c>
       <c r="K45" s="17" t="n">
-        <v>0.41834486</v>
+        <v>0</v>
       </c>
       <c r="L45" s="11" t="n"/>
       <c r="M45" s="20" t="n">
@@ -2428,10 +2428,10 @@
         <v>85000</v>
       </c>
       <c r="J48" s="18" t="n">
-        <v>85000</v>
+        <v>0</v>
       </c>
       <c r="K48" s="17" t="n">
-        <v>0.02370621</v>
+        <v>0</v>
       </c>
       <c r="L48" s="11" t="n"/>
       <c r="M48" s="20" t="n">
@@ -2472,10 +2472,10 @@
         <v>85000</v>
       </c>
       <c r="J49" s="18" t="n">
-        <v>85000</v>
+        <v>0</v>
       </c>
       <c r="K49" s="17" t="n">
-        <v>0.02370621</v>
+        <v>0</v>
       </c>
       <c r="L49" s="11" t="n"/>
       <c r="M49" s="20" t="n">
@@ -2572,10 +2572,10 @@
         <v>5500</v>
       </c>
       <c r="J52" s="18" t="n">
-        <v>1140625.2</v>
+        <v>0</v>
       </c>
       <c r="K52" s="17" t="n">
-        <v>0.31811646</v>
+        <v>0</v>
       </c>
       <c r="L52" s="11" t="n"/>
       <c r="M52" s="20" t="n">
@@ -2618,10 +2618,10 @@
         <v>255550</v>
       </c>
       <c r="J53" s="18" t="n">
-        <v>52997594.52</v>
+        <v>0</v>
       </c>
       <c r="K53" s="17" t="n">
-        <v>14.78084761</v>
+        <v>0</v>
       </c>
       <c r="L53" s="11" t="n"/>
       <c r="M53" s="17" t="n"/>
@@ -2668,10 +2668,10 @@
         <v>26853</v>
       </c>
       <c r="J54" s="18" t="n">
-        <v>2684225.88</v>
+        <v>0</v>
       </c>
       <c r="K54" s="17" t="n">
-        <v>0.74862141</v>
+        <v>0</v>
       </c>
       <c r="L54" s="11" t="n"/>
       <c r="M54" s="17" t="n"/>
@@ -2718,10 +2718,10 @@
         <v>61335</v>
       </c>
       <c r="J55" s="18" t="n">
-        <v>9363401.1</v>
+        <v>0</v>
       </c>
       <c r="K55" s="17" t="n">
-        <v>2.6114205</v>
+        <v>0</v>
       </c>
       <c r="L55" s="11" t="n"/>
       <c r="M55" s="17" t="n"/>
@@ -2768,10 +2768,10 @@
         <v>449902</v>
       </c>
       <c r="J56" s="18" t="n">
-        <v>5398824</v>
+        <v>0</v>
       </c>
       <c r="K56" s="17" t="n">
-        <v>1.50571352</v>
+        <v>0</v>
       </c>
       <c r="L56" s="11" t="n"/>
       <c r="M56" s="20" t="n">
@@ -2814,10 +2814,10 @@
         <v>668187</v>
       </c>
       <c r="J57" s="18" t="n">
-        <v>8018244</v>
+        <v>0</v>
       </c>
       <c r="K57" s="17" t="n">
-        <v>2.23626079</v>
+        <v>0</v>
       </c>
       <c r="L57" s="11" t="n"/>
       <c r="M57" s="17" t="n"/>
@@ -2864,10 +2864,10 @@
         <v>63699</v>
       </c>
       <c r="J58" s="18" t="n">
-        <v>191097</v>
+        <v>0</v>
       </c>
       <c r="K58" s="17" t="n">
-        <v>0.0532963</v>
+        <v>0</v>
       </c>
       <c r="L58" s="11" t="n"/>
       <c r="M58" s="17" t="n"/>
@@ -2970,10 +2970,10 @@
         <v>5500</v>
       </c>
       <c r="J61" s="18" t="n">
-        <v>791076</v>
+        <v>0</v>
       </c>
       <c r="K61" s="17" t="n">
-        <v>0.22062839</v>
+        <v>0</v>
       </c>
       <c r="L61" s="11" t="n"/>
       <c r="M61" s="20" t="n">
@@ -3016,10 +3016,10 @@
         <v>255550</v>
       </c>
       <c r="J62" s="18" t="n">
-        <v>36756267.6</v>
+        <v>0</v>
       </c>
       <c r="K62" s="17" t="n">
-        <v>10.25119715</v>
+        <v>0</v>
       </c>
       <c r="L62" s="11" t="n"/>
       <c r="M62" s="17" t="n"/>
@@ -3066,10 +3066,10 @@
         <v>26853</v>
       </c>
       <c r="J63" s="18" t="n">
-        <v>1828152.24</v>
+        <v>0</v>
       </c>
       <c r="K63" s="17" t="n">
-        <v>0.5098654</v>
+        <v>0</v>
       </c>
       <c r="L63" s="11" t="n"/>
       <c r="M63" s="17" t="n"/>
@@ -3116,10 +3116,10 @@
         <v>61335</v>
       </c>
       <c r="J64" s="18" t="n">
-        <v>6016350.15</v>
+        <v>0</v>
       </c>
       <c r="K64" s="17" t="n">
-        <v>1.67793945</v>
+        <v>0</v>
       </c>
       <c r="L64" s="11" t="n"/>
       <c r="M64" s="17" t="n"/>
@@ -3166,10 +3166,10 @@
         <v>449902</v>
       </c>
       <c r="J65" s="18" t="n">
-        <v>3599216</v>
+        <v>0</v>
       </c>
       <c r="K65" s="17" t="n">
-        <v>1.00380902</v>
+        <v>0</v>
       </c>
       <c r="L65" s="11" t="n"/>
       <c r="M65" s="20" t="n">
@@ -3212,10 +3212,10 @@
         <v>668187</v>
       </c>
       <c r="J66" s="18" t="n">
-        <v>5345496</v>
+        <v>0</v>
       </c>
       <c r="K66" s="17" t="n">
-        <v>1.49084053</v>
+        <v>0</v>
       </c>
       <c r="L66" s="11" t="n"/>
       <c r="M66" s="17" t="n"/>
@@ -3262,10 +3262,10 @@
         <v>63699</v>
       </c>
       <c r="J67" s="18" t="n">
-        <v>127398</v>
+        <v>0</v>
       </c>
       <c r="K67" s="17" t="n">
-        <v>0.03553087</v>
+        <v>0</v>
       </c>
       <c r="L67" s="11" t="n"/>
       <c r="M67" s="17" t="n"/>
@@ -3400,10 +3400,10 @@
         <v>5500</v>
       </c>
       <c r="J71" s="18" t="n">
-        <v>27610</v>
+        <v>0</v>
       </c>
       <c r="K71" s="17" t="n">
-        <v>0.00770033</v>
+        <v>0</v>
       </c>
       <c r="L71" s="11" t="n"/>
       <c r="M71" s="17" t="n"/>
@@ -3444,10 +3444,10 @@
         <v>255550</v>
       </c>
       <c r="J72" s="18" t="n">
-        <v>1282861</v>
+        <v>0</v>
       </c>
       <c r="K72" s="17" t="n">
-        <v>0.35778554</v>
+        <v>0</v>
       </c>
       <c r="L72" s="11" t="n"/>
       <c r="M72" s="17" t="n"/>
@@ -3490,10 +3490,10 @@
         <v>26853</v>
       </c>
       <c r="J73" s="18" t="n">
-        <v>341033.1</v>
+        <v>0</v>
       </c>
       <c r="K73" s="17" t="n">
-        <v>0.09511296</v>
+        <v>0</v>
       </c>
       <c r="L73" s="11" t="n"/>
       <c r="M73" s="17" t="n"/>
@@ -3536,10 +3536,10 @@
         <v>61335</v>
       </c>
       <c r="J74" s="18" t="n">
-        <v>122670</v>
+        <v>0</v>
       </c>
       <c r="K74" s="17" t="n">
-        <v>0.03421224</v>
+        <v>0</v>
       </c>
       <c r="L74" s="11" t="n"/>
       <c r="M74" s="17" t="n"/>
@@ -3582,10 +3582,10 @@
         <v>449902</v>
       </c>
       <c r="J75" s="18" t="n">
-        <v>899804</v>
+        <v>0</v>
       </c>
       <c r="K75" s="17" t="n">
-        <v>0.25095225</v>
+        <v>0</v>
       </c>
       <c r="L75" s="11" t="n"/>
       <c r="M75" s="17" t="n"/>
@@ -3628,10 +3628,10 @@
         <v>63699</v>
       </c>
       <c r="J76" s="18" t="n">
-        <v>127398</v>
+        <v>0</v>
       </c>
       <c r="K76" s="17" t="n">
-        <v>0.03553087</v>
+        <v>0</v>
       </c>
       <c r="L76" s="11" t="n"/>
       <c r="M76" s="17" t="n"/>
@@ -3730,10 +3730,10 @@
         <v>97486</v>
       </c>
       <c r="J79" s="18" t="n">
-        <v>1131081.315</v>
+        <v>0</v>
       </c>
       <c r="K79" s="17" t="n">
-        <v>0.31545471</v>
+        <v>0</v>
       </c>
       <c r="L79" s="11" t="n"/>
       <c r="M79" s="20" t="n">
@@ -3774,10 +3774,10 @@
         <v>5500</v>
       </c>
       <c r="J80" s="18" t="n">
-        <v>746620.875</v>
+        <v>0</v>
       </c>
       <c r="K80" s="17" t="n">
-        <v>0.20823001</v>
+        <v>0</v>
       </c>
       <c r="L80" s="11" t="n"/>
       <c r="M80" s="20" t="n">
@@ -3818,10 +3818,10 @@
         <v>255550</v>
       </c>
       <c r="J81" s="18" t="n">
-        <v>34690720.8375</v>
+        <v>0</v>
       </c>
       <c r="K81" s="17" t="n">
-        <v>9.675123230000001</v>
+        <v>0</v>
       </c>
       <c r="L81" s="11" t="n"/>
       <c r="M81" s="17" t="n"/>
@@ -3866,10 +3866,10 @@
         <v>26853</v>
       </c>
       <c r="J82" s="18" t="n">
-        <v>1773372.12</v>
+        <v>0</v>
       </c>
       <c r="K82" s="17" t="n">
-        <v>0.49458741</v>
+        <v>0</v>
       </c>
       <c r="L82" s="11" t="n"/>
       <c r="M82" s="17" t="n"/>
@@ -3912,10 +3912,10 @@
         <v>61335</v>
       </c>
       <c r="J83" s="18" t="n">
-        <v>9923389.65</v>
+        <v>0</v>
       </c>
       <c r="K83" s="17" t="n">
-        <v>2.76759939</v>
+        <v>0</v>
       </c>
       <c r="L83" s="11" t="n"/>
       <c r="M83" s="17" t="n"/>
@@ -3960,10 +3960,10 @@
         <v>449902</v>
       </c>
       <c r="J84" s="18" t="n">
-        <v>3599216</v>
+        <v>0</v>
       </c>
       <c r="K84" s="17" t="n">
-        <v>1.00380902</v>
+        <v>0</v>
       </c>
       <c r="L84" s="11" t="n"/>
       <c r="M84" s="17" t="n"/>
@@ -4006,10 +4006,10 @@
         <v>668187</v>
       </c>
       <c r="J85" s="18" t="n">
-        <v>5345496</v>
+        <v>0</v>
       </c>
       <c r="K85" s="17" t="n">
-        <v>1.49084053</v>
+        <v>0</v>
       </c>
       <c r="L85" s="11" t="n"/>
       <c r="M85" s="17" t="n"/>
@@ -4052,10 +4052,10 @@
         <v>63699</v>
       </c>
       <c r="J86" s="18" t="n">
-        <v>127398</v>
+        <v>0</v>
       </c>
       <c r="K86" s="17" t="n">
-        <v>0.03553087</v>
+        <v>0</v>
       </c>
       <c r="L86" s="11" t="n"/>
       <c r="M86" s="17" t="n"/>
@@ -4138,7 +4138,7 @@
       </c>
       <c r="C89" s="14" t="inlineStr">
         <is>
-          <t>Lantai 1</t>
+          <t>Lantai 2</t>
         </is>
       </c>
       <c r="D89" s="33" t="n"/>
@@ -4186,10 +4186,10 @@
         <v>5500</v>
       </c>
       <c r="J90" s="18" t="n">
-        <v>2277976.8</v>
+        <v>0</v>
       </c>
       <c r="K90" s="17" t="n">
-        <v>0.63531993</v>
+        <v>0</v>
       </c>
       <c r="L90" s="11" t="n"/>
       <c r="M90" s="17" t="n"/>
@@ -4230,10 +4230,10 @@
         <v>255550</v>
       </c>
       <c r="J91" s="18" t="n">
-        <v>61584381.18</v>
+        <v>0</v>
       </c>
       <c r="K91" s="17" t="n">
-        <v>17.175673</v>
+        <v>0</v>
       </c>
       <c r="L91" s="11" t="n"/>
       <c r="M91" s="17" t="n"/>
@@ -4282,10 +4282,10 @@
         <v>277206</v>
       </c>
       <c r="J92" s="18" t="n">
-        <v>48009307.14</v>
+        <v>0</v>
       </c>
       <c r="K92" s="17" t="n">
-        <v>13.38963134</v>
+        <v>0</v>
       </c>
       <c r="L92" s="11" t="n"/>
       <c r="M92" s="17" t="n"/>
@@ -4334,10 +4334,10 @@
         <v>26853</v>
       </c>
       <c r="J93" s="18" t="n">
-        <v>3335142.6</v>
+        <v>0</v>
       </c>
       <c r="K93" s="17" t="n">
-        <v>0.93015985</v>
+        <v>0</v>
       </c>
       <c r="L93" s="11" t="n"/>
       <c r="M93" s="17" t="n"/>
@@ -4386,10 +4386,10 @@
         <v>26853</v>
       </c>
       <c r="J94" s="18" t="n">
-        <v>5735263.74</v>
+        <v>0</v>
       </c>
       <c r="K94" s="17" t="n">
-        <v>1.59954542</v>
+        <v>0</v>
       </c>
       <c r="L94" s="11" t="n"/>
       <c r="M94" s="17" t="n"/>
@@ -4438,10 +4438,10 @@
         <v>449902</v>
       </c>
       <c r="J95" s="18" t="n">
-        <v>17546178</v>
+        <v>0</v>
       </c>
       <c r="K95" s="17" t="n">
-        <v>4.89356895</v>
+        <v>0</v>
       </c>
       <c r="L95" s="11" t="n"/>
       <c r="M95" s="17" t="n"/>
@@ -4486,10 +4486,10 @@
         <v>244459</v>
       </c>
       <c r="J96" s="18" t="n">
-        <v>3666885</v>
+        <v>0</v>
       </c>
       <c r="K96" s="17" t="n">
-        <v>1.02268167</v>
+        <v>0</v>
       </c>
       <c r="L96" s="11" t="n"/>
       <c r="M96" s="17" t="n"/>
@@ -4532,10 +4532,10 @@
         <v>668187</v>
       </c>
       <c r="J97" s="18" t="n">
-        <v>16036488</v>
+        <v>0</v>
       </c>
       <c r="K97" s="17" t="n">
-        <v>4.47252158</v>
+        <v>0</v>
       </c>
       <c r="L97" s="11" t="n"/>
       <c r="M97" s="17" t="n"/>
@@ -4578,10 +4578,10 @@
         <v>63699</v>
       </c>
       <c r="J98" s="18" t="n">
-        <v>254796</v>
+        <v>0</v>
       </c>
       <c r="K98" s="17" t="n">
-        <v>0.07106173</v>
+        <v>0</v>
       </c>
       <c r="L98" s="11" t="n"/>
       <c r="M98" s="17" t="n"/>
@@ -4624,10 +4624,10 @@
         <v>46759</v>
       </c>
       <c r="J99" s="18" t="n">
-        <v>93518</v>
+        <v>0</v>
       </c>
       <c r="K99" s="17" t="n">
-        <v>0.02608185</v>
+        <v>0</v>
       </c>
       <c r="L99" s="11" t="n"/>
       <c r="M99" s="17" t="n"/>
@@ -5293,7 +5293,7 @@
         <v>2.312</v>
       </c>
       <c r="C2" s="52" t="n">
-        <v>0</v>
+        <v>7.06</v>
       </c>
       <c r="F2" t="n">
         <v>21</v>
@@ -5309,7 +5309,7 @@
         <v>8.943</v>
       </c>
       <c r="C3" s="52" t="n">
-        <v>0</v>
+        <v>9.726000000000001</v>
       </c>
       <c r="F3" t="n">
         <v>25</v>
@@ -5325,7 +5325,7 @@
         <v>25.422</v>
       </c>
       <c r="C4" s="52" t="n">
-        <v>0</v>
+        <v>9.726000000000001</v>
       </c>
       <c r="F4" t="n">
         <v>99</v>
@@ -5341,7 +5341,7 @@
         <v>55.025</v>
       </c>
       <c r="C5" s="52" t="n">
-        <v>0</v>
+        <v>9.726000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -5354,7 +5354,7 @@
         <v>72.816</v>
       </c>
       <c r="C6" s="52" t="n">
-        <v>0</v>
+        <v>9.726000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -5367,7 +5367,7 @@
         <v>83.726</v>
       </c>
       <c r="C7" s="52" t="n">
-        <v>0</v>
+        <v>9.726000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -5380,7 +5380,7 @@
         <v>94.53700000000001</v>
       </c>
       <c r="C8" s="52" t="n">
-        <v>0</v>
+        <v>9.726000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -5393,7 +5393,7 @@
         <v>98.81</v>
       </c>
       <c r="C9" s="52" t="n">
-        <v>0</v>
+        <v>9.726000000000001</v>
       </c>
     </row>
     <row r="10">
@@ -5406,7 +5406,7 @@
         <v>100</v>
       </c>
       <c r="C10" s="52" t="n">
-        <v>0</v>
+        <v>9.726000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adendum versi satu done
</commit_message>
<xml_diff>
--- a/backend/final_schedule.xlsx
+++ b/backend/final_schedule.xlsx
@@ -1096,7 +1096,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>RP 397.997.000</t>
+          <t>RP 397.997</t>
         </is>
       </c>
     </row>
@@ -1608,39 +1608,29 @@
         <v>1999280</v>
       </c>
       <c r="J29" s="18" t="n">
-        <v>0</v>
+        <v>1999280</v>
       </c>
       <c r="K29" s="17" t="n">
-        <v>0</v>
+        <v>0.557592</v>
       </c>
       <c r="L29" s="11" t="n"/>
       <c r="M29" s="20" t="n">
-        <v>0.0619547</v>
+        <v>0.06195467</v>
       </c>
       <c r="N29" s="20" t="n">
-        <v>0.0619547</v>
+        <v>0.06195467</v>
       </c>
       <c r="O29" s="20" t="n">
-        <v>0.0619547</v>
+        <v>0.06195467</v>
       </c>
       <c r="P29" s="20" t="n">
-        <v>0.0619547</v>
-      </c>
-      <c r="Q29" s="20" t="n">
-        <v>0.0619547</v>
-      </c>
-      <c r="R29" s="20" t="n">
-        <v>0.0619547</v>
-      </c>
-      <c r="S29" s="20" t="n">
-        <v>0.0619547</v>
-      </c>
-      <c r="T29" s="20" t="n">
-        <v>0.0619547</v>
-      </c>
-      <c r="U29" s="20" t="n">
-        <v>0.0619547</v>
-      </c>
+        <v>0.06195467</v>
+      </c>
+      <c r="Q29" s="17" t="n"/>
+      <c r="R29" s="17" t="n"/>
+      <c r="S29" s="17" t="n"/>
+      <c r="T29" s="17" t="n"/>
+      <c r="U29" s="17" t="n"/>
       <c r="V29" s="11" t="n"/>
       <c r="W29" s="19" t="n"/>
     </row>
@@ -1724,39 +1714,29 @@
         <v>300000</v>
       </c>
       <c r="J32" s="18" t="n">
-        <v>0</v>
+        <v>300000</v>
       </c>
       <c r="K32" s="17" t="n">
-        <v>0</v>
+        <v>0.08366899999999999</v>
       </c>
       <c r="L32" s="11" t="n"/>
       <c r="M32" s="20" t="n">
-        <v>0.009296550000000001</v>
+        <v>0.009296560000000001</v>
       </c>
       <c r="N32" s="20" t="n">
-        <v>0.009296550000000001</v>
+        <v>0.009296560000000001</v>
       </c>
       <c r="O32" s="20" t="n">
-        <v>0.009296550000000001</v>
+        <v>0.009296560000000001</v>
       </c>
       <c r="P32" s="20" t="n">
-        <v>0.009296550000000001</v>
-      </c>
-      <c r="Q32" s="20" t="n">
-        <v>0.009296550000000001</v>
-      </c>
-      <c r="R32" s="20" t="n">
-        <v>0.009296550000000001</v>
-      </c>
-      <c r="S32" s="20" t="n">
-        <v>0.009296550000000001</v>
-      </c>
-      <c r="T32" s="20" t="n">
-        <v>0.009296550000000001</v>
-      </c>
-      <c r="U32" s="20" t="n">
-        <v>0.009296550000000001</v>
-      </c>
+        <v>0.009296560000000001</v>
+      </c>
+      <c r="Q32" s="17" t="n"/>
+      <c r="R32" s="17" t="n"/>
+      <c r="S32" s="17" t="n"/>
+      <c r="T32" s="17" t="n"/>
+      <c r="U32" s="17" t="n"/>
       <c r="V32" s="11" t="n"/>
       <c r="W32" s="19" t="n"/>
     </row>
@@ -1784,39 +1764,29 @@
         <v>150000</v>
       </c>
       <c r="J33" s="18" t="n">
-        <v>0</v>
+        <v>150000</v>
       </c>
       <c r="K33" s="17" t="n">
-        <v>0</v>
+        <v>0.041834</v>
       </c>
       <c r="L33" s="11" t="n"/>
       <c r="M33" s="20" t="n">
-        <v>0.00464828</v>
+        <v>0.00464822</v>
       </c>
       <c r="N33" s="20" t="n">
-        <v>0.00464828</v>
+        <v>0.00464822</v>
       </c>
       <c r="O33" s="20" t="n">
-        <v>0.00464828</v>
+        <v>0.00464822</v>
       </c>
       <c r="P33" s="20" t="n">
-        <v>0.00464828</v>
-      </c>
-      <c r="Q33" s="20" t="n">
-        <v>0.00464828</v>
-      </c>
-      <c r="R33" s="20" t="n">
-        <v>0.00464828</v>
-      </c>
-      <c r="S33" s="20" t="n">
-        <v>0.00464828</v>
-      </c>
-      <c r="T33" s="20" t="n">
-        <v>0.00464828</v>
-      </c>
-      <c r="U33" s="20" t="n">
-        <v>0.00464828</v>
-      </c>
+        <v>0.00464822</v>
+      </c>
+      <c r="Q33" s="17" t="n"/>
+      <c r="R33" s="17" t="n"/>
+      <c r="S33" s="17" t="n"/>
+      <c r="T33" s="17" t="n"/>
+      <c r="U33" s="17" t="n"/>
       <c r="V33" s="11" t="n"/>
       <c r="W33" s="19" t="n"/>
     </row>
@@ -1900,10 +1870,10 @@
         <v>25000</v>
       </c>
       <c r="J36" s="18" t="n">
-        <v>0</v>
+        <v>125000</v>
       </c>
       <c r="K36" s="17" t="n">
-        <v>0</v>
+        <v>0.034862</v>
       </c>
       <c r="L36" s="11" t="n"/>
       <c r="M36" s="20" t="n">
@@ -1918,21 +1888,11 @@
       <c r="P36" s="20" t="n">
         <v>0.00387356</v>
       </c>
-      <c r="Q36" s="20" t="n">
-        <v>0.00387356</v>
-      </c>
-      <c r="R36" s="20" t="n">
-        <v>0.00387356</v>
-      </c>
-      <c r="S36" s="20" t="n">
-        <v>0.00387356</v>
-      </c>
-      <c r="T36" s="20" t="n">
-        <v>0.00387356</v>
-      </c>
-      <c r="U36" s="20" t="n">
-        <v>0.00387356</v>
-      </c>
+      <c r="Q36" s="17" t="n"/>
+      <c r="R36" s="17" t="n"/>
+      <c r="S36" s="17" t="n"/>
+      <c r="T36" s="17" t="n"/>
+      <c r="U36" s="17" t="n"/>
       <c r="V36" s="11" t="n"/>
       <c r="W36" s="19" t="n"/>
     </row>
@@ -1960,39 +1920,29 @@
         <v>60000</v>
       </c>
       <c r="J37" s="18" t="n">
-        <v>0</v>
+        <v>60000</v>
       </c>
       <c r="K37" s="17" t="n">
-        <v>0</v>
+        <v>0.016734</v>
       </c>
       <c r="L37" s="11" t="n"/>
       <c r="M37" s="20" t="n">
-        <v>0.00185931</v>
+        <v>0.00185933</v>
       </c>
       <c r="N37" s="20" t="n">
-        <v>0.00185931</v>
+        <v>0.00185933</v>
       </c>
       <c r="O37" s="20" t="n">
-        <v>0.00185931</v>
+        <v>0.00185933</v>
       </c>
       <c r="P37" s="20" t="n">
-        <v>0.00185931</v>
-      </c>
-      <c r="Q37" s="20" t="n">
-        <v>0.00185931</v>
-      </c>
-      <c r="R37" s="20" t="n">
-        <v>0.00185931</v>
-      </c>
-      <c r="S37" s="20" t="n">
-        <v>0.00185931</v>
-      </c>
-      <c r="T37" s="20" t="n">
-        <v>0.00185931</v>
-      </c>
-      <c r="U37" s="20" t="n">
-        <v>0.00185931</v>
-      </c>
+        <v>0.00185933</v>
+      </c>
+      <c r="Q37" s="17" t="n"/>
+      <c r="R37" s="17" t="n"/>
+      <c r="S37" s="17" t="n"/>
+      <c r="T37" s="17" t="n"/>
+      <c r="U37" s="17" t="n"/>
       <c r="V37" s="11" t="n"/>
       <c r="W37" s="19" t="n"/>
     </row>
@@ -2020,39 +1970,29 @@
         <v>68000</v>
       </c>
       <c r="J38" s="18" t="n">
-        <v>0</v>
+        <v>340000</v>
       </c>
       <c r="K38" s="17" t="n">
-        <v>0</v>
+        <v>0.09482500000000001</v>
       </c>
       <c r="L38" s="11" t="n"/>
       <c r="M38" s="20" t="n">
-        <v>0.01053609</v>
+        <v>0.01053611</v>
       </c>
       <c r="N38" s="20" t="n">
-        <v>0.01053609</v>
+        <v>0.01053611</v>
       </c>
       <c r="O38" s="20" t="n">
-        <v>0.01053609</v>
+        <v>0.01053611</v>
       </c>
       <c r="P38" s="20" t="n">
-        <v>0.01053609</v>
-      </c>
-      <c r="Q38" s="20" t="n">
-        <v>0.01053609</v>
-      </c>
-      <c r="R38" s="20" t="n">
-        <v>0.01053609</v>
-      </c>
-      <c r="S38" s="20" t="n">
-        <v>0.01053609</v>
-      </c>
-      <c r="T38" s="20" t="n">
-        <v>0.01053609</v>
-      </c>
-      <c r="U38" s="20" t="n">
-        <v>0.01053609</v>
-      </c>
+        <v>0.01053611</v>
+      </c>
+      <c r="Q38" s="17" t="n"/>
+      <c r="R38" s="17" t="n"/>
+      <c r="S38" s="17" t="n"/>
+      <c r="T38" s="17" t="n"/>
+      <c r="U38" s="17" t="n"/>
       <c r="V38" s="11" t="n"/>
       <c r="W38" s="19" t="n"/>
     </row>
@@ -2080,39 +2020,29 @@
         <v>35000</v>
       </c>
       <c r="J39" s="18" t="n">
-        <v>0</v>
+        <v>175000</v>
       </c>
       <c r="K39" s="17" t="n">
-        <v>0</v>
+        <v>0.048807</v>
       </c>
       <c r="L39" s="11" t="n"/>
       <c r="M39" s="20" t="n">
-        <v>0.00542299</v>
+        <v>0.005423</v>
       </c>
       <c r="N39" s="20" t="n">
-        <v>0.00542299</v>
+        <v>0.005423</v>
       </c>
       <c r="O39" s="20" t="n">
-        <v>0.00542299</v>
+        <v>0.005423</v>
       </c>
       <c r="P39" s="20" t="n">
-        <v>0.00542299</v>
-      </c>
-      <c r="Q39" s="20" t="n">
-        <v>0.00542299</v>
-      </c>
-      <c r="R39" s="20" t="n">
-        <v>0.00542299</v>
-      </c>
-      <c r="S39" s="20" t="n">
-        <v>0.00542299</v>
-      </c>
-      <c r="T39" s="20" t="n">
-        <v>0.00542299</v>
-      </c>
-      <c r="U39" s="20" t="n">
-        <v>0.00542299</v>
-      </c>
+        <v>0.005423</v>
+      </c>
+      <c r="Q39" s="17" t="n"/>
+      <c r="R39" s="17" t="n"/>
+      <c r="S39" s="17" t="n"/>
+      <c r="T39" s="17" t="n"/>
+      <c r="U39" s="17" t="n"/>
       <c r="V39" s="11" t="n"/>
       <c r="W39" s="19" t="n"/>
     </row>
@@ -2196,39 +2126,29 @@
         <v>800000</v>
       </c>
       <c r="J42" s="18" t="n">
-        <v>0</v>
+        <v>800000</v>
       </c>
       <c r="K42" s="17" t="n">
-        <v>0</v>
+        <v>0.223117</v>
       </c>
       <c r="L42" s="11" t="n"/>
       <c r="M42" s="20" t="n">
-        <v>0.02479081</v>
+        <v>0.02479078</v>
       </c>
       <c r="N42" s="20" t="n">
-        <v>0.02479081</v>
+        <v>0.02479078</v>
       </c>
       <c r="O42" s="20" t="n">
-        <v>0.02479081</v>
+        <v>0.02479078</v>
       </c>
       <c r="P42" s="20" t="n">
-        <v>0.02479081</v>
-      </c>
-      <c r="Q42" s="20" t="n">
-        <v>0.02479081</v>
-      </c>
-      <c r="R42" s="20" t="n">
-        <v>0.02479081</v>
-      </c>
-      <c r="S42" s="20" t="n">
-        <v>0.02479081</v>
-      </c>
-      <c r="T42" s="20" t="n">
-        <v>0.02479081</v>
-      </c>
-      <c r="U42" s="20" t="n">
-        <v>0.02479081</v>
-      </c>
+        <v>0.02479078</v>
+      </c>
+      <c r="Q42" s="17" t="n"/>
+      <c r="R42" s="17" t="n"/>
+      <c r="S42" s="17" t="n"/>
+      <c r="T42" s="17" t="n"/>
+      <c r="U42" s="17" t="n"/>
       <c r="V42" s="11" t="n"/>
       <c r="W42" s="19" t="n"/>
     </row>
@@ -2312,39 +2232,29 @@
         <v>1500000</v>
       </c>
       <c r="J45" s="18" t="n">
-        <v>0</v>
+        <v>1500000</v>
       </c>
       <c r="K45" s="17" t="n">
-        <v>0</v>
+        <v>0.418345</v>
       </c>
       <c r="L45" s="11" t="n"/>
       <c r="M45" s="20" t="n">
-        <v>0.04648276</v>
+        <v>0.04648278</v>
       </c>
       <c r="N45" s="20" t="n">
-        <v>0.04648276</v>
+        <v>0.04648278</v>
       </c>
       <c r="O45" s="20" t="n">
-        <v>0.04648276</v>
+        <v>0.04648278</v>
       </c>
       <c r="P45" s="20" t="n">
-        <v>0.04648276</v>
-      </c>
-      <c r="Q45" s="20" t="n">
-        <v>0.04648276</v>
-      </c>
-      <c r="R45" s="20" t="n">
-        <v>0.04648276</v>
-      </c>
-      <c r="S45" s="20" t="n">
-        <v>0.04648276</v>
-      </c>
-      <c r="T45" s="20" t="n">
-        <v>0.04648276</v>
-      </c>
-      <c r="U45" s="20" t="n">
-        <v>0.04648276</v>
-      </c>
+        <v>0.04648278</v>
+      </c>
+      <c r="Q45" s="17" t="n"/>
+      <c r="R45" s="17" t="n"/>
+      <c r="S45" s="17" t="n"/>
+      <c r="T45" s="17" t="n"/>
+      <c r="U45" s="17" t="n"/>
       <c r="V45" s="11" t="n"/>
       <c r="W45" s="19" t="n"/>
     </row>
@@ -2428,14 +2338,14 @@
         <v>85000</v>
       </c>
       <c r="J48" s="18" t="n">
-        <v>0</v>
+        <v>85000</v>
       </c>
       <c r="K48" s="17" t="n">
-        <v>0</v>
+        <v>0.023706</v>
       </c>
       <c r="L48" s="11" t="n"/>
       <c r="M48" s="20" t="n">
-        <v>0.02370621</v>
+        <v>0.023706</v>
       </c>
       <c r="N48" s="17" t="n"/>
       <c r="O48" s="17" t="n"/>
@@ -2472,14 +2382,14 @@
         <v>85000</v>
       </c>
       <c r="J49" s="18" t="n">
-        <v>0</v>
+        <v>85000</v>
       </c>
       <c r="K49" s="17" t="n">
-        <v>0</v>
+        <v>0.023706</v>
       </c>
       <c r="L49" s="11" t="n"/>
       <c r="M49" s="20" t="n">
-        <v>0.02370621</v>
+        <v>0.023706</v>
       </c>
       <c r="N49" s="17" t="n"/>
       <c r="O49" s="17" t="n"/>
@@ -2566,23 +2476,23 @@
         </is>
       </c>
       <c r="H52" s="17" t="n">
-        <v>207.3864</v>
+        <v>215.34</v>
       </c>
       <c r="I52" s="18" t="n">
         <v>5500</v>
       </c>
       <c r="J52" s="18" t="n">
-        <v>0</v>
+        <v>1184370</v>
       </c>
       <c r="K52" s="17" t="n">
-        <v>0</v>
+        <v>0.330317</v>
       </c>
       <c r="L52" s="11" t="n"/>
       <c r="M52" s="20" t="n">
-        <v>0.15905823</v>
+        <v>0.159058</v>
       </c>
       <c r="N52" s="20" t="n">
-        <v>0.15905823</v>
+        <v>0.159058</v>
       </c>
       <c r="O52" s="17" t="n"/>
       <c r="P52" s="17" t="n"/>
@@ -2612,32 +2522,28 @@
         </is>
       </c>
       <c r="H53" s="17" t="n">
-        <v>207.3864</v>
+        <v>215.34</v>
       </c>
       <c r="I53" s="18" t="n">
         <v>255550</v>
       </c>
       <c r="J53" s="18" t="n">
-        <v>0</v>
+        <v>55030137</v>
       </c>
       <c r="K53" s="17" t="n">
-        <v>0</v>
+        <v>15.347717</v>
       </c>
       <c r="L53" s="11" t="n"/>
       <c r="M53" s="17" t="n"/>
       <c r="N53" s="17" t="n"/>
       <c r="O53" s="20" t="n">
-        <v>3.6952119</v>
+        <v>3.695212</v>
       </c>
       <c r="P53" s="20" t="n">
-        <v>3.6952119</v>
-      </c>
-      <c r="Q53" s="20" t="n">
-        <v>3.6952119</v>
-      </c>
-      <c r="R53" s="20" t="n">
-        <v>3.6952119</v>
-      </c>
+        <v>3.695212</v>
+      </c>
+      <c r="Q53" s="17" t="n"/>
+      <c r="R53" s="17" t="n"/>
       <c r="S53" s="17" t="n"/>
       <c r="T53" s="17" t="n"/>
       <c r="U53" s="17" t="n"/>
@@ -2662,32 +2568,28 @@
         </is>
       </c>
       <c r="H54" s="17" t="n">
-        <v>99.95999999999999</v>
+        <v>102.06</v>
       </c>
       <c r="I54" s="18" t="n">
         <v>26853</v>
       </c>
       <c r="J54" s="18" t="n">
-        <v>0</v>
+        <v>2740617.18</v>
       </c>
       <c r="K54" s="17" t="n">
-        <v>0</v>
+        <v>0.7643489999999999</v>
       </c>
       <c r="L54" s="11" t="n"/>
       <c r="M54" s="17" t="n"/>
       <c r="N54" s="17" t="n"/>
       <c r="O54" s="20" t="n">
-        <v>0.18715535</v>
+        <v>0.18715525</v>
       </c>
       <c r="P54" s="20" t="n">
-        <v>0.18715535</v>
-      </c>
-      <c r="Q54" s="20" t="n">
-        <v>0.18715535</v>
-      </c>
-      <c r="R54" s="20" t="n">
-        <v>0.18715535</v>
-      </c>
+        <v>0.18715525</v>
+      </c>
+      <c r="Q54" s="17" t="n"/>
+      <c r="R54" s="17" t="n"/>
       <c r="S54" s="17" t="n"/>
       <c r="T54" s="17" t="n"/>
       <c r="U54" s="17" t="n"/>
@@ -2718,25 +2620,23 @@
         <v>61335</v>
       </c>
       <c r="J55" s="18" t="n">
-        <v>0</v>
+        <v>9363401.1</v>
       </c>
       <c r="K55" s="17" t="n">
-        <v>0</v>
+        <v>2.61142</v>
       </c>
       <c r="L55" s="11" t="n"/>
       <c r="M55" s="17" t="n"/>
       <c r="N55" s="20" t="n">
-        <v>0.65285512</v>
+        <v>0.652855</v>
       </c>
       <c r="O55" s="20" t="n">
-        <v>0.65285512</v>
+        <v>0.652855</v>
       </c>
       <c r="P55" s="20" t="n">
-        <v>0.65285512</v>
-      </c>
-      <c r="Q55" s="20" t="n">
-        <v>0.65285512</v>
-      </c>
+        <v>0.652855</v>
+      </c>
+      <c r="Q55" s="17" t="n"/>
       <c r="R55" s="17" t="n"/>
       <c r="S55" s="17" t="n"/>
       <c r="T55" s="17" t="n"/>
@@ -2762,7 +2662,7 @@
         </is>
       </c>
       <c r="H56" s="17" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="I56" s="18" t="n">
         <v>449902</v>
@@ -2775,10 +2675,10 @@
       </c>
       <c r="L56" s="11" t="n"/>
       <c r="M56" s="20" t="n">
-        <v>0.75285676</v>
+        <v>0.752857</v>
       </c>
       <c r="N56" s="20" t="n">
-        <v>0.75285676</v>
+        <v>0.752857</v>
       </c>
       <c r="O56" s="17" t="n"/>
       <c r="P56" s="17" t="n"/>
@@ -2814,28 +2714,20 @@
         <v>668187</v>
       </c>
       <c r="J57" s="18" t="n">
-        <v>0</v>
+        <v>8018244</v>
       </c>
       <c r="K57" s="17" t="n">
-        <v>0</v>
+        <v>2.236261</v>
       </c>
       <c r="L57" s="11" t="n"/>
       <c r="M57" s="17" t="n"/>
       <c r="N57" s="17" t="n"/>
       <c r="O57" s="17" t="n"/>
       <c r="P57" s="17" t="n"/>
-      <c r="Q57" s="20" t="n">
-        <v>0.5590652</v>
-      </c>
-      <c r="R57" s="20" t="n">
-        <v>0.5590652</v>
-      </c>
-      <c r="S57" s="20" t="n">
-        <v>0.5590652</v>
-      </c>
-      <c r="T57" s="20" t="n">
-        <v>0.5590652</v>
-      </c>
+      <c r="Q57" s="17" t="n"/>
+      <c r="R57" s="17" t="n"/>
+      <c r="S57" s="17" t="n"/>
+      <c r="T57" s="17" t="n"/>
       <c r="U57" s="17" t="n"/>
       <c r="V57" s="11" t="n"/>
       <c r="W57" s="19" t="n"/>
@@ -2864,28 +2756,20 @@
         <v>63699</v>
       </c>
       <c r="J58" s="18" t="n">
-        <v>0</v>
+        <v>191097</v>
       </c>
       <c r="K58" s="17" t="n">
-        <v>0</v>
+        <v>0.053296</v>
       </c>
       <c r="L58" s="11" t="n"/>
       <c r="M58" s="17" t="n"/>
       <c r="N58" s="17" t="n"/>
       <c r="O58" s="17" t="n"/>
       <c r="P58" s="17" t="n"/>
-      <c r="Q58" s="20" t="n">
-        <v>0.01332407</v>
-      </c>
-      <c r="R58" s="20" t="n">
-        <v>0.01332407</v>
-      </c>
-      <c r="S58" s="20" t="n">
-        <v>0.01332407</v>
-      </c>
-      <c r="T58" s="20" t="n">
-        <v>0.01332407</v>
-      </c>
+      <c r="Q58" s="17" t="n"/>
+      <c r="R58" s="17" t="n"/>
+      <c r="S58" s="17" t="n"/>
+      <c r="T58" s="17" t="n"/>
       <c r="U58" s="17" t="n"/>
       <c r="V58" s="11" t="n"/>
       <c r="W58" s="19" t="n"/>
@@ -2970,17 +2854,17 @@
         <v>5500</v>
       </c>
       <c r="J61" s="18" t="n">
-        <v>0</v>
+        <v>791076</v>
       </c>
       <c r="K61" s="17" t="n">
-        <v>0</v>
+        <v>0.220628</v>
       </c>
       <c r="L61" s="11" t="n"/>
       <c r="M61" s="20" t="n">
-        <v>0.1103142</v>
+        <v>0.110314</v>
       </c>
       <c r="N61" s="20" t="n">
-        <v>0.1103142</v>
+        <v>0.110314</v>
       </c>
       <c r="O61" s="17" t="n"/>
       <c r="P61" s="17" t="n"/>
@@ -3016,26 +2900,22 @@
         <v>255550</v>
       </c>
       <c r="J62" s="18" t="n">
-        <v>0</v>
+        <v>36756267.6</v>
       </c>
       <c r="K62" s="17" t="n">
-        <v>0</v>
+        <v>10.251197</v>
       </c>
       <c r="L62" s="11" t="n"/>
       <c r="M62" s="17" t="n"/>
       <c r="N62" s="17" t="n"/>
       <c r="O62" s="20" t="n">
-        <v>1.70853286</v>
+        <v>1.70853283</v>
       </c>
       <c r="P62" s="20" t="n">
-        <v>3.41706572</v>
-      </c>
-      <c r="Q62" s="20" t="n">
-        <v>3.41706572</v>
-      </c>
-      <c r="R62" s="20" t="n">
-        <v>1.70853285</v>
-      </c>
+        <v>3.41706567</v>
+      </c>
+      <c r="Q62" s="17" t="n"/>
+      <c r="R62" s="17" t="n"/>
       <c r="S62" s="17" t="n"/>
       <c r="T62" s="17" t="n"/>
       <c r="U62" s="17" t="n"/>
@@ -3066,26 +2946,22 @@
         <v>26853</v>
       </c>
       <c r="J63" s="18" t="n">
-        <v>0</v>
+        <v>1828152.24</v>
       </c>
       <c r="K63" s="17" t="n">
-        <v>0</v>
+        <v>0.509865</v>
       </c>
       <c r="L63" s="11" t="n"/>
       <c r="M63" s="17" t="n"/>
       <c r="N63" s="17" t="n"/>
       <c r="O63" s="20" t="n">
-        <v>0.12746635</v>
+        <v>0.12746625</v>
       </c>
       <c r="P63" s="20" t="n">
-        <v>0.12746635</v>
-      </c>
-      <c r="Q63" s="20" t="n">
-        <v>0.12746635</v>
-      </c>
-      <c r="R63" s="20" t="n">
-        <v>0.12746635</v>
-      </c>
+        <v>0.12746625</v>
+      </c>
+      <c r="Q63" s="17" t="n"/>
+      <c r="R63" s="17" t="n"/>
       <c r="S63" s="17" t="n"/>
       <c r="T63" s="17" t="n"/>
       <c r="U63" s="17" t="n"/>
@@ -3116,10 +2992,10 @@
         <v>61335</v>
       </c>
       <c r="J64" s="18" t="n">
-        <v>0</v>
+        <v>6016350.15</v>
       </c>
       <c r="K64" s="17" t="n">
-        <v>0</v>
+        <v>1.677939</v>
       </c>
       <c r="L64" s="11" t="n"/>
       <c r="M64" s="17" t="n"/>
@@ -3132,9 +3008,7 @@
       <c r="P64" s="20" t="n">
         <v>0.5159792</v>
       </c>
-      <c r="Q64" s="20" t="n">
-        <v>0.13000185</v>
-      </c>
+      <c r="Q64" s="17" t="n"/>
       <c r="R64" s="17" t="n"/>
       <c r="S64" s="17" t="n"/>
       <c r="T64" s="17" t="n"/>
@@ -3160,7 +3034,7 @@
         </is>
       </c>
       <c r="H65" s="17" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="I65" s="18" t="n">
         <v>449902</v>
@@ -3176,7 +3050,7 @@
         <v>0.55015167</v>
       </c>
       <c r="N65" s="20" t="n">
-        <v>0.45365735</v>
+        <v>0.45365733</v>
       </c>
       <c r="O65" s="17" t="n"/>
       <c r="P65" s="17" t="n"/>
@@ -3212,28 +3086,20 @@
         <v>668187</v>
       </c>
       <c r="J66" s="18" t="n">
-        <v>0</v>
+        <v>5345496</v>
       </c>
       <c r="K66" s="17" t="n">
-        <v>0</v>
+        <v>1.490841</v>
       </c>
       <c r="L66" s="11" t="n"/>
       <c r="M66" s="17" t="n"/>
       <c r="N66" s="17" t="n"/>
       <c r="O66" s="17" t="n"/>
       <c r="P66" s="17" t="n"/>
-      <c r="Q66" s="20" t="n">
-        <v>0.37271013</v>
-      </c>
-      <c r="R66" s="20" t="n">
-        <v>0.37271013</v>
-      </c>
-      <c r="S66" s="20" t="n">
-        <v>0.37271013</v>
-      </c>
-      <c r="T66" s="20" t="n">
-        <v>0.37271013</v>
-      </c>
+      <c r="Q66" s="17" t="n"/>
+      <c r="R66" s="17" t="n"/>
+      <c r="S66" s="17" t="n"/>
+      <c r="T66" s="17" t="n"/>
       <c r="U66" s="17" t="n"/>
       <c r="V66" s="11" t="n"/>
       <c r="W66" s="19" t="n"/>
@@ -3262,28 +3128,20 @@
         <v>63699</v>
       </c>
       <c r="J67" s="18" t="n">
-        <v>0</v>
+        <v>127398</v>
       </c>
       <c r="K67" s="17" t="n">
-        <v>0</v>
+        <v>0.035531</v>
       </c>
       <c r="L67" s="11" t="n"/>
       <c r="M67" s="17" t="n"/>
       <c r="N67" s="17" t="n"/>
       <c r="O67" s="17" t="n"/>
       <c r="P67" s="17" t="n"/>
-      <c r="Q67" s="20" t="n">
-        <v>0.00888272</v>
-      </c>
-      <c r="R67" s="20" t="n">
-        <v>0.00888272</v>
-      </c>
-      <c r="S67" s="20" t="n">
-        <v>0.00888272</v>
-      </c>
-      <c r="T67" s="20" t="n">
-        <v>0.00888272</v>
-      </c>
+      <c r="Q67" s="17" t="n"/>
+      <c r="R67" s="17" t="n"/>
+      <c r="S67" s="17" t="n"/>
+      <c r="T67" s="17" t="n"/>
       <c r="U67" s="17" t="n"/>
       <c r="V67" s="11" t="n"/>
       <c r="W67" s="19" t="n"/>
@@ -3400,10 +3258,10 @@
         <v>5500</v>
       </c>
       <c r="J71" s="18" t="n">
-        <v>0</v>
+        <v>27610</v>
       </c>
       <c r="K71" s="17" t="n">
-        <v>0</v>
+        <v>0.0077</v>
       </c>
       <c r="L71" s="11" t="n"/>
       <c r="M71" s="17" t="n"/>
@@ -3413,9 +3271,7 @@
       <c r="Q71" s="17" t="n"/>
       <c r="R71" s="17" t="n"/>
       <c r="S71" s="17" t="n"/>
-      <c r="T71" s="20" t="n">
-        <v>0.00770033</v>
-      </c>
+      <c r="T71" s="17" t="n"/>
       <c r="U71" s="17" t="n"/>
       <c r="V71" s="11" t="n"/>
       <c r="W71" s="19" t="n"/>
@@ -3444,10 +3300,10 @@
         <v>255550</v>
       </c>
       <c r="J72" s="18" t="n">
-        <v>0</v>
+        <v>1282861</v>
       </c>
       <c r="K72" s="17" t="n">
-        <v>0</v>
+        <v>0.357786</v>
       </c>
       <c r="L72" s="11" t="n"/>
       <c r="M72" s="17" t="n"/>
@@ -3457,12 +3313,8 @@
       <c r="Q72" s="17" t="n"/>
       <c r="R72" s="17" t="n"/>
       <c r="S72" s="17" t="n"/>
-      <c r="T72" s="20" t="n">
-        <v>0.23852369</v>
-      </c>
-      <c r="U72" s="20" t="n">
-        <v>0.11926185</v>
-      </c>
+      <c r="T72" s="17" t="n"/>
+      <c r="U72" s="17" t="n"/>
       <c r="V72" s="11" t="n"/>
       <c r="W72" s="19" t="n"/>
     </row>
@@ -3490,10 +3342,10 @@
         <v>26853</v>
       </c>
       <c r="J73" s="18" t="n">
-        <v>0</v>
+        <v>341033.1</v>
       </c>
       <c r="K73" s="17" t="n">
-        <v>0</v>
+        <v>0.095113</v>
       </c>
       <c r="L73" s="11" t="n"/>
       <c r="M73" s="17" t="n"/>
@@ -3503,12 +3355,8 @@
       <c r="Q73" s="17" t="n"/>
       <c r="R73" s="17" t="n"/>
       <c r="S73" s="17" t="n"/>
-      <c r="T73" s="20" t="n">
-        <v>0.06340864</v>
-      </c>
-      <c r="U73" s="20" t="n">
-        <v>0.03170432</v>
-      </c>
+      <c r="T73" s="17" t="n"/>
+      <c r="U73" s="17" t="n"/>
       <c r="V73" s="11" t="n"/>
       <c r="W73" s="19" t="n"/>
     </row>
@@ -3536,10 +3384,10 @@
         <v>61335</v>
       </c>
       <c r="J74" s="18" t="n">
-        <v>0</v>
+        <v>122670</v>
       </c>
       <c r="K74" s="17" t="n">
-        <v>0</v>
+        <v>0.034212</v>
       </c>
       <c r="L74" s="11" t="n"/>
       <c r="M74" s="17" t="n"/>
@@ -3549,12 +3397,8 @@
       <c r="Q74" s="17" t="n"/>
       <c r="R74" s="17" t="n"/>
       <c r="S74" s="17" t="n"/>
-      <c r="T74" s="20" t="n">
-        <v>0.02280816</v>
-      </c>
-      <c r="U74" s="20" t="n">
-        <v>0.01140408</v>
-      </c>
+      <c r="T74" s="17" t="n"/>
+      <c r="U74" s="17" t="n"/>
       <c r="V74" s="11" t="n"/>
       <c r="W74" s="19" t="n"/>
     </row>
@@ -3582,10 +3426,10 @@
         <v>449902</v>
       </c>
       <c r="J75" s="18" t="n">
-        <v>0</v>
+        <v>899804</v>
       </c>
       <c r="K75" s="17" t="n">
-        <v>0</v>
+        <v>0.250952</v>
       </c>
       <c r="L75" s="11" t="n"/>
       <c r="M75" s="17" t="n"/>
@@ -3595,12 +3439,8 @@
       <c r="Q75" s="17" t="n"/>
       <c r="R75" s="17" t="n"/>
       <c r="S75" s="17" t="n"/>
-      <c r="T75" s="20" t="n">
-        <v>0.1673015</v>
-      </c>
-      <c r="U75" s="20" t="n">
-        <v>0.08365075</v>
-      </c>
+      <c r="T75" s="17" t="n"/>
+      <c r="U75" s="17" t="n"/>
       <c r="V75" s="11" t="n"/>
       <c r="W75" s="19" t="n"/>
     </row>
@@ -3628,10 +3468,10 @@
         <v>63699</v>
       </c>
       <c r="J76" s="18" t="n">
-        <v>0</v>
+        <v>127398</v>
       </c>
       <c r="K76" s="17" t="n">
-        <v>0</v>
+        <v>0.035531</v>
       </c>
       <c r="L76" s="11" t="n"/>
       <c r="M76" s="17" t="n"/>
@@ -3641,12 +3481,8 @@
       <c r="Q76" s="17" t="n"/>
       <c r="R76" s="17" t="n"/>
       <c r="S76" s="17" t="n"/>
-      <c r="T76" s="20" t="n">
-        <v>0.02368725</v>
-      </c>
-      <c r="U76" s="20" t="n">
-        <v>0.01184362</v>
-      </c>
+      <c r="T76" s="17" t="n"/>
+      <c r="U76" s="17" t="n"/>
       <c r="V76" s="11" t="n"/>
       <c r="W76" s="19" t="n"/>
     </row>
@@ -3730,14 +3566,14 @@
         <v>97486</v>
       </c>
       <c r="J79" s="18" t="n">
-        <v>0</v>
+        <v>1131081.315</v>
       </c>
       <c r="K79" s="17" t="n">
-        <v>0</v>
+        <v>0.315455</v>
       </c>
       <c r="L79" s="11" t="n"/>
       <c r="M79" s="20" t="n">
-        <v>0.31545471</v>
+        <v>0.315455</v>
       </c>
       <c r="N79" s="17" t="n"/>
       <c r="O79" s="17" t="n"/>
@@ -3768,20 +3604,20 @@
         </is>
       </c>
       <c r="H80" s="17" t="n">
-        <v>135.74925</v>
+        <v>67.87462499999999</v>
       </c>
       <c r="I80" s="18" t="n">
         <v>5500</v>
       </c>
       <c r="J80" s="18" t="n">
-        <v>0</v>
+        <v>373310.4374999999</v>
       </c>
       <c r="K80" s="17" t="n">
-        <v>0</v>
+        <v>0.104115</v>
       </c>
       <c r="L80" s="11" t="n"/>
       <c r="M80" s="20" t="n">
-        <v>0.20823001</v>
+        <v>0.20823</v>
       </c>
       <c r="N80" s="17" t="n"/>
       <c r="O80" s="17" t="n"/>
@@ -3812,27 +3648,27 @@
         </is>
       </c>
       <c r="H81" s="17" t="n">
-        <v>135.74925</v>
+        <v>67.87462499999999</v>
       </c>
       <c r="I81" s="18" t="n">
         <v>255550</v>
       </c>
       <c r="J81" s="18" t="n">
-        <v>0</v>
+        <v>17345360.41875</v>
       </c>
       <c r="K81" s="17" t="n">
-        <v>0</v>
+        <v>4.837562</v>
       </c>
       <c r="L81" s="11" t="n"/>
       <c r="M81" s="17" t="n"/>
       <c r="N81" s="20" t="n">
-        <v>1.2093904</v>
+        <v>1.20939038</v>
       </c>
       <c r="O81" s="20" t="n">
-        <v>4.7893144</v>
+        <v>4.78931444</v>
       </c>
       <c r="P81" s="20" t="n">
-        <v>3.67641843</v>
+        <v>3.67641818</v>
       </c>
       <c r="Q81" s="17" t="n"/>
       <c r="R81" s="17" t="n"/>
@@ -3860,24 +3696,24 @@
         </is>
       </c>
       <c r="H82" s="17" t="n">
-        <v>66.04000000000001</v>
+        <v>33.02</v>
       </c>
       <c r="I82" s="18" t="n">
         <v>26853</v>
       </c>
       <c r="J82" s="18" t="n">
-        <v>0</v>
+        <v>886686.0600000001</v>
       </c>
       <c r="K82" s="17" t="n">
-        <v>0</v>
+        <v>0.247294</v>
       </c>
       <c r="L82" s="11" t="n"/>
       <c r="M82" s="17" t="n"/>
       <c r="N82" s="20" t="n">
-        <v>0.24729371</v>
+        <v>0.2472935</v>
       </c>
       <c r="O82" s="20" t="n">
-        <v>0.24729371</v>
+        <v>0.2472935</v>
       </c>
       <c r="P82" s="17" t="n"/>
       <c r="Q82" s="17" t="n"/>
@@ -3912,25 +3748,19 @@
         <v>61335</v>
       </c>
       <c r="J83" s="18" t="n">
-        <v>0</v>
+        <v>9923389.65</v>
       </c>
       <c r="K83" s="17" t="n">
-        <v>0</v>
+        <v>2.767599</v>
       </c>
       <c r="L83" s="11" t="n"/>
       <c r="M83" s="17" t="n"/>
       <c r="N83" s="17" t="n"/>
       <c r="O83" s="17" t="n"/>
       <c r="P83" s="17" t="n"/>
-      <c r="Q83" s="20" t="n">
-        <v>0.18450663</v>
-      </c>
-      <c r="R83" s="20" t="n">
-        <v>0.34594992</v>
-      </c>
-      <c r="S83" s="20" t="n">
-        <v>2.23714284</v>
-      </c>
+      <c r="Q83" s="17" t="n"/>
+      <c r="R83" s="17" t="n"/>
+      <c r="S83" s="17" t="n"/>
       <c r="T83" s="17" t="n"/>
       <c r="U83" s="17" t="n"/>
       <c r="V83" s="11" t="n"/>
@@ -3954,7 +3784,7 @@
         </is>
       </c>
       <c r="H84" s="17" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="I84" s="18" t="n">
         <v>449902</v>
@@ -3968,10 +3798,10 @@
       <c r="L84" s="11" t="n"/>
       <c r="M84" s="17" t="n"/>
       <c r="N84" s="20" t="n">
-        <v>0.50190451</v>
+        <v>0.5019045</v>
       </c>
       <c r="O84" s="20" t="n">
-        <v>0.50190451</v>
+        <v>0.5019045</v>
       </c>
       <c r="P84" s="17" t="n"/>
       <c r="Q84" s="17" t="n"/>
@@ -4000,16 +3830,16 @@
         </is>
       </c>
       <c r="H85" s="17" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I85" s="18" t="n">
         <v>668187</v>
       </c>
       <c r="J85" s="18" t="n">
-        <v>0</v>
+        <v>2672748</v>
       </c>
       <c r="K85" s="17" t="n">
-        <v>0</v>
+        <v>0.74542</v>
       </c>
       <c r="L85" s="11" t="n"/>
       <c r="M85" s="17" t="n"/>
@@ -4019,12 +3849,8 @@
       <c r="Q85" s="17" t="n"/>
       <c r="R85" s="17" t="n"/>
       <c r="S85" s="17" t="n"/>
-      <c r="T85" s="20" t="n">
-        <v>0.74542027</v>
-      </c>
-      <c r="U85" s="20" t="n">
-        <v>0.74542027</v>
-      </c>
+      <c r="T85" s="17" t="n"/>
+      <c r="U85" s="17" t="n"/>
       <c r="V85" s="11" t="n"/>
       <c r="W85" s="19" t="n"/>
     </row>
@@ -4046,16 +3872,16 @@
         </is>
       </c>
       <c r="H86" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I86" s="18" t="n">
         <v>63699</v>
       </c>
       <c r="J86" s="18" t="n">
-        <v>0</v>
+        <v>63699</v>
       </c>
       <c r="K86" s="17" t="n">
-        <v>0</v>
+        <v>0.017765</v>
       </c>
       <c r="L86" s="11" t="n"/>
       <c r="M86" s="17" t="n"/>
@@ -4065,12 +3891,8 @@
       <c r="Q86" s="17" t="n"/>
       <c r="R86" s="17" t="n"/>
       <c r="S86" s="17" t="n"/>
-      <c r="T86" s="20" t="n">
-        <v>0.01776544</v>
-      </c>
-      <c r="U86" s="20" t="n">
-        <v>0.01776544</v>
-      </c>
+      <c r="T86" s="17" t="n"/>
+      <c r="U86" s="17" t="n"/>
       <c r="V86" s="11" t="n"/>
       <c r="W86" s="19" t="n"/>
     </row>
@@ -4138,7 +3960,7 @@
       </c>
       <c r="C89" s="14" t="inlineStr">
         <is>
-          <t>Lantai 2</t>
+          <t>Lantai 1</t>
         </is>
       </c>
       <c r="D89" s="33" t="n"/>
@@ -4180,21 +4002,21 @@
         </is>
       </c>
       <c r="H90" s="17" t="n">
-        <v>414.1776</v>
+        <v>572.822</v>
       </c>
       <c r="I90" s="18" t="n">
         <v>5500</v>
       </c>
       <c r="J90" s="18" t="n">
-        <v>0</v>
+        <v>3150521</v>
       </c>
       <c r="K90" s="17" t="n">
-        <v>0</v>
+        <v>0.87867</v>
       </c>
       <c r="L90" s="11" t="n"/>
       <c r="M90" s="17" t="n"/>
       <c r="N90" s="20" t="n">
-        <v>0.63531993</v>
+        <v>0.63532</v>
       </c>
       <c r="O90" s="17" t="n"/>
       <c r="P90" s="17" t="n"/>
@@ -4224,16 +4046,16 @@
         </is>
       </c>
       <c r="H91" s="17" t="n">
-        <v>240.9876</v>
+        <v>297.18</v>
       </c>
       <c r="I91" s="18" t="n">
         <v>255550</v>
       </c>
       <c r="J91" s="18" t="n">
-        <v>0</v>
+        <v>75944349</v>
       </c>
       <c r="K91" s="17" t="n">
-        <v>0</v>
+        <v>21.180619</v>
       </c>
       <c r="L91" s="11" t="n"/>
       <c r="M91" s="17" t="n"/>
@@ -4244,15 +4066,9 @@
       <c r="P91" s="20" t="n">
         <v>5.18136414</v>
       </c>
-      <c r="Q91" s="20" t="n">
-        <v>4.29391825</v>
-      </c>
-      <c r="R91" s="20" t="n">
-        <v>3.37309326</v>
-      </c>
-      <c r="S91" s="20" t="n">
-        <v>3.37309329</v>
-      </c>
+      <c r="Q91" s="17" t="n"/>
+      <c r="R91" s="17" t="n"/>
+      <c r="S91" s="17" t="n"/>
       <c r="T91" s="17" t="n"/>
       <c r="U91" s="17" t="n"/>
       <c r="V91" s="11" t="n"/>
@@ -4276,35 +4092,29 @@
         </is>
       </c>
       <c r="H92" s="17" t="n">
-        <v>173.19</v>
+        <v>275.642</v>
       </c>
       <c r="I92" s="18" t="n">
         <v>277206</v>
       </c>
       <c r="J92" s="18" t="n">
-        <v>0</v>
+        <v>76409616.252</v>
       </c>
       <c r="K92" s="17" t="n">
-        <v>0</v>
+        <v>21.31038</v>
       </c>
       <c r="L92" s="11" t="n"/>
       <c r="M92" s="17" t="n"/>
       <c r="N92" s="17" t="n"/>
       <c r="O92" s="20" t="n">
-        <v>0.74386841</v>
+        <v>0.74386839</v>
       </c>
       <c r="P92" s="20" t="n">
-        <v>9.23160521</v>
-      </c>
-      <c r="Q92" s="20" t="n">
-        <v>3.34740784</v>
-      </c>
-      <c r="R92" s="20" t="n">
-        <v>0.03337494</v>
-      </c>
-      <c r="S92" s="20" t="n">
-        <v>0.03337494</v>
-      </c>
+        <v>9.231605220000001</v>
+      </c>
+      <c r="Q92" s="17" t="n"/>
+      <c r="R92" s="17" t="n"/>
+      <c r="S92" s="17" t="n"/>
       <c r="T92" s="17" t="n"/>
       <c r="U92" s="17" t="n"/>
       <c r="V92" s="11" t="n"/>
@@ -4328,35 +4138,29 @@
         </is>
       </c>
       <c r="H93" s="17" t="n">
-        <v>124.2</v>
+        <v>154.2</v>
       </c>
       <c r="I93" s="18" t="n">
         <v>26853</v>
       </c>
       <c r="J93" s="18" t="n">
-        <v>0</v>
+        <v>4140732.6</v>
       </c>
       <c r="K93" s="17" t="n">
-        <v>0</v>
+        <v>1.154836</v>
       </c>
       <c r="L93" s="11" t="n"/>
       <c r="M93" s="17" t="n"/>
       <c r="N93" s="17" t="n"/>
       <c r="O93" s="20" t="n">
-        <v>0.15502664</v>
+        <v>0.15502667</v>
       </c>
       <c r="P93" s="20" t="n">
-        <v>0.31005328</v>
-      </c>
-      <c r="Q93" s="20" t="n">
-        <v>0.23253996</v>
-      </c>
-      <c r="R93" s="20" t="n">
-        <v>0.11626999</v>
-      </c>
-      <c r="S93" s="20" t="n">
-        <v>0.11626999</v>
-      </c>
+        <v>0.31005333</v>
+      </c>
+      <c r="Q93" s="17" t="n"/>
+      <c r="R93" s="17" t="n"/>
+      <c r="S93" s="17" t="n"/>
       <c r="T93" s="17" t="n"/>
       <c r="U93" s="17" t="n"/>
       <c r="V93" s="11" t="n"/>
@@ -4380,35 +4184,29 @@
         </is>
       </c>
       <c r="H94" s="17" t="n">
-        <v>213.58</v>
+        <v>267.6554554</v>
       </c>
       <c r="I94" s="18" t="n">
         <v>26853</v>
       </c>
       <c r="J94" s="18" t="n">
-        <v>0</v>
+        <v>7187351.9438562</v>
       </c>
       <c r="K94" s="17" t="n">
-        <v>0</v>
+        <v>2.004528</v>
       </c>
       <c r="L94" s="11" t="n"/>
       <c r="M94" s="17" t="n"/>
       <c r="N94" s="17" t="n"/>
       <c r="O94" s="20" t="n">
-        <v>0.39988636</v>
+        <v>0.39988625</v>
       </c>
       <c r="P94" s="20" t="n">
-        <v>0.39988636</v>
-      </c>
-      <c r="Q94" s="20" t="n">
-        <v>0.39988636</v>
-      </c>
-      <c r="R94" s="20" t="n">
-        <v>0.19994317</v>
-      </c>
-      <c r="S94" s="20" t="n">
-        <v>0.19994317</v>
-      </c>
+        <v>0.39988625</v>
+      </c>
+      <c r="Q94" s="17" t="n"/>
+      <c r="R94" s="17" t="n"/>
+      <c r="S94" s="17" t="n"/>
       <c r="T94" s="17" t="n"/>
       <c r="U94" s="17" t="n"/>
       <c r="V94" s="11" t="n"/>
@@ -4432,27 +4230,27 @@
         </is>
       </c>
       <c r="H95" s="17" t="n">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="I95" s="18" t="n">
         <v>449902</v>
       </c>
       <c r="J95" s="18" t="n">
-        <v>0</v>
+        <v>6298628</v>
       </c>
       <c r="K95" s="17" t="n">
-        <v>0</v>
+        <v>1.756666</v>
       </c>
       <c r="L95" s="11" t="n"/>
       <c r="M95" s="17" t="n"/>
       <c r="N95" s="20" t="n">
-        <v>1.22339224</v>
+        <v>1.22339225</v>
       </c>
       <c r="O95" s="20" t="n">
-        <v>1.63118965</v>
+        <v>1.63118967</v>
       </c>
       <c r="P95" s="20" t="n">
-        <v>2.03898706</v>
+        <v>2.03898708</v>
       </c>
       <c r="Q95" s="17" t="n"/>
       <c r="R95" s="17" t="n"/>
@@ -4480,16 +4278,16 @@
         </is>
       </c>
       <c r="H96" s="17" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I96" s="18" t="n">
         <v>244459</v>
       </c>
       <c r="J96" s="18" t="n">
-        <v>0</v>
+        <v>3422426</v>
       </c>
       <c r="K96" s="17" t="n">
-        <v>0</v>
+        <v>0.954503</v>
       </c>
       <c r="L96" s="11" t="n"/>
       <c r="M96" s="17" t="n"/>
@@ -4498,12 +4296,8 @@
       <c r="P96" s="17" t="n"/>
       <c r="Q96" s="17" t="n"/>
       <c r="R96" s="17" t="n"/>
-      <c r="S96" s="20" t="n">
-        <v>0.68178778</v>
-      </c>
-      <c r="T96" s="20" t="n">
-        <v>0.34089389</v>
-      </c>
+      <c r="S96" s="17" t="n"/>
+      <c r="T96" s="17" t="n"/>
       <c r="U96" s="17" t="n"/>
       <c r="V96" s="11" t="n"/>
       <c r="W96" s="19" t="n"/>
@@ -4526,16 +4320,16 @@
         </is>
       </c>
       <c r="H97" s="17" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="I97" s="18" t="n">
         <v>668187</v>
       </c>
       <c r="J97" s="18" t="n">
-        <v>0</v>
+        <v>13363740</v>
       </c>
       <c r="K97" s="17" t="n">
-        <v>0</v>
+        <v>3.727101</v>
       </c>
       <c r="L97" s="11" t="n"/>
       <c r="M97" s="17" t="n"/>
@@ -4544,12 +4338,8 @@
       <c r="P97" s="17" t="n"/>
       <c r="Q97" s="17" t="n"/>
       <c r="R97" s="17" t="n"/>
-      <c r="S97" s="20" t="n">
-        <v>2.98168105</v>
-      </c>
-      <c r="T97" s="20" t="n">
-        <v>1.49084053</v>
-      </c>
+      <c r="S97" s="17" t="n"/>
+      <c r="T97" s="17" t="n"/>
       <c r="U97" s="17" t="n"/>
       <c r="V97" s="11" t="n"/>
       <c r="W97" s="19" t="n"/>
@@ -4572,16 +4362,16 @@
         </is>
       </c>
       <c r="H98" s="17" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I98" s="18" t="n">
         <v>63699</v>
       </c>
       <c r="J98" s="18" t="n">
-        <v>0</v>
+        <v>382194</v>
       </c>
       <c r="K98" s="17" t="n">
-        <v>0</v>
+        <v>0.106593</v>
       </c>
       <c r="L98" s="11" t="n"/>
       <c r="M98" s="17" t="n"/>
@@ -4590,12 +4380,8 @@
       <c r="P98" s="17" t="n"/>
       <c r="Q98" s="17" t="n"/>
       <c r="R98" s="17" t="n"/>
-      <c r="S98" s="20" t="n">
-        <v>0.04737449</v>
-      </c>
-      <c r="T98" s="20" t="n">
-        <v>0.02368724</v>
-      </c>
+      <c r="S98" s="17" t="n"/>
+      <c r="T98" s="17" t="n"/>
       <c r="U98" s="17" t="n"/>
       <c r="V98" s="11" t="n"/>
       <c r="W98" s="19" t="n"/>
@@ -4618,16 +4404,16 @@
         </is>
       </c>
       <c r="H99" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I99" s="18" t="n">
         <v>46759</v>
       </c>
       <c r="J99" s="18" t="n">
-        <v>0</v>
+        <v>46759</v>
       </c>
       <c r="K99" s="17" t="n">
-        <v>0</v>
+        <v>0.013041</v>
       </c>
       <c r="L99" s="11" t="n"/>
       <c r="M99" s="17" t="n"/>
@@ -4636,12 +4422,8 @@
       <c r="P99" s="17" t="n"/>
       <c r="Q99" s="17" t="n"/>
       <c r="R99" s="17" t="n"/>
-      <c r="S99" s="20" t="n">
-        <v>0.0173879</v>
-      </c>
-      <c r="T99" s="20" t="n">
-        <v>0.008693950000000001</v>
-      </c>
+      <c r="S99" s="17" t="n"/>
+      <c r="T99" s="17" t="n"/>
       <c r="U99" s="17" t="n"/>
       <c r="V99" s="11" t="n"/>
       <c r="W99" s="19" t="n"/>
@@ -5293,7 +5075,7 @@
         <v>2.312</v>
       </c>
       <c r="C2" s="52" t="n">
-        <v>7.06</v>
+        <v>7.252</v>
       </c>
       <c r="F2" t="n">
         <v>21</v>
@@ -5309,7 +5091,7 @@
         <v>8.943</v>
       </c>
       <c r="C3" s="52" t="n">
-        <v>9.726000000000001</v>
+        <v>10.05</v>
       </c>
       <c r="F3" t="n">
         <v>25</v>
@@ -5325,7 +5107,7 @@
         <v>25.422</v>
       </c>
       <c r="C4" s="52" t="n">
-        <v>9.726000000000001</v>
+        <v>28.684</v>
       </c>
       <c r="F4" t="n">
         <v>99</v>
@@ -5341,7 +5123,7 @@
         <v>55.025</v>
       </c>
       <c r="C5" s="52" t="n">
-        <v>9.726000000000001</v>
+        <v>77.035</v>
       </c>
     </row>
     <row r="6">
@@ -5351,10 +5133,10 @@
         </is>
       </c>
       <c r="B6" s="52" t="n">
-        <v>72.816</v>
+        <v>55.025</v>
       </c>
       <c r="C6" s="52" t="n">
-        <v>9.726000000000001</v>
+        <v>73.06100000000001</v>
       </c>
     </row>
     <row r="7">
@@ -5364,10 +5146,10 @@
         </is>
       </c>
       <c r="B7" s="52" t="n">
-        <v>83.726</v>
+        <v>55.025</v>
       </c>
       <c r="C7" s="52" t="n">
-        <v>9.726000000000001</v>
+        <v>73.06100000000001</v>
       </c>
     </row>
     <row r="8">
@@ -5377,10 +5159,10 @@
         </is>
       </c>
       <c r="B8" s="52" t="n">
-        <v>94.53700000000001</v>
+        <v>55.025</v>
       </c>
       <c r="C8" s="52" t="n">
-        <v>9.726000000000001</v>
+        <v>73.06100000000001</v>
       </c>
     </row>
     <row r="9">
@@ -5390,10 +5172,10 @@
         </is>
       </c>
       <c r="B9" s="52" t="n">
-        <v>98.81</v>
+        <v>55.025</v>
       </c>
       <c r="C9" s="52" t="n">
-        <v>9.726000000000001</v>
+        <v>73.06100000000001</v>
       </c>
     </row>
     <row r="10">
@@ -5403,10 +5185,10 @@
         </is>
       </c>
       <c r="B10" s="52" t="n">
-        <v>100</v>
+        <v>55.025</v>
       </c>
       <c r="C10" s="52" t="n">
-        <v>9.726000000000001</v>
+        <v>73.06100000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update schaduel lihat presisi
</commit_message>
<xml_diff>
--- a/backend/final_schedule.xlsx
+++ b/backend/final_schedule.xlsx
@@ -1583,31 +1583,31 @@
       </c>
       <c r="L29" s="11" t="n"/>
       <c r="M29" s="20" t="n">
-        <v>0.06195467</v>
+        <v>0.062</v>
       </c>
       <c r="N29" s="20" t="n">
-        <v>0.06195467</v>
+        <v>0.062</v>
       </c>
       <c r="O29" s="20" t="n">
-        <v>0.06195467</v>
+        <v>0.062</v>
       </c>
       <c r="P29" s="20" t="n">
-        <v>0.06195467</v>
+        <v>0.062</v>
       </c>
       <c r="Q29" s="20" t="n">
-        <v>0.06195467</v>
+        <v>0.062</v>
       </c>
       <c r="R29" s="20" t="n">
-        <v>0.06195467</v>
+        <v>0.062</v>
       </c>
       <c r="S29" s="20" t="n">
-        <v>0.06195467</v>
+        <v>0.062</v>
       </c>
       <c r="T29" s="20" t="n">
-        <v>0.06195467</v>
+        <v>0.062</v>
       </c>
       <c r="U29" s="20" t="n">
-        <v>0.06195467</v>
+        <v>0.062</v>
       </c>
       <c r="V29" s="11" t="n"/>
       <c r="W29" s="19" t="n"/>
@@ -1699,31 +1699,31 @@
       </c>
       <c r="L32" s="11" t="n"/>
       <c r="M32" s="20" t="n">
-        <v>0.009296560000000001</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="N32" s="20" t="n">
-        <v>0.009296560000000001</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="O32" s="20" t="n">
-        <v>0.009296560000000001</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="P32" s="20" t="n">
-        <v>0.009296560000000001</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>0.009296560000000001</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="R32" s="20" t="n">
-        <v>0.009296560000000001</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="S32" s="20" t="n">
-        <v>0.009296560000000001</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="T32" s="20" t="n">
-        <v>0.009296560000000001</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="U32" s="20" t="n">
-        <v>0.009296560000000001</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="V32" s="11" t="n"/>
       <c r="W32" s="19" t="n"/>
@@ -1759,31 +1759,31 @@
       </c>
       <c r="L33" s="11" t="n"/>
       <c r="M33" s="20" t="n">
-        <v>0.00464822</v>
+        <v>0.0046</v>
       </c>
       <c r="N33" s="20" t="n">
-        <v>0.00464822</v>
+        <v>0.0046</v>
       </c>
       <c r="O33" s="20" t="n">
-        <v>0.00464822</v>
+        <v>0.0046</v>
       </c>
       <c r="P33" s="20" t="n">
-        <v>0.00464822</v>
+        <v>0.0046</v>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>0.00464822</v>
+        <v>0.0046</v>
       </c>
       <c r="R33" s="20" t="n">
-        <v>0.00464822</v>
+        <v>0.0046</v>
       </c>
       <c r="S33" s="20" t="n">
-        <v>0.00464822</v>
+        <v>0.0046</v>
       </c>
       <c r="T33" s="20" t="n">
-        <v>0.00464822</v>
+        <v>0.0046</v>
       </c>
       <c r="U33" s="20" t="n">
-        <v>0.00464822</v>
+        <v>0.0046</v>
       </c>
       <c r="V33" s="11" t="n"/>
       <c r="W33" s="19" t="n"/>
@@ -1875,31 +1875,31 @@
       </c>
       <c r="L36" s="11" t="n"/>
       <c r="M36" s="20" t="n">
-        <v>0.00387356</v>
+        <v>0.0039</v>
       </c>
       <c r="N36" s="20" t="n">
-        <v>0.00387356</v>
+        <v>0.0039</v>
       </c>
       <c r="O36" s="20" t="n">
-        <v>0.00387356</v>
+        <v>0.0039</v>
       </c>
       <c r="P36" s="20" t="n">
-        <v>0.00387356</v>
+        <v>0.0039</v>
       </c>
       <c r="Q36" s="20" t="n">
-        <v>0.00387356</v>
+        <v>0.0039</v>
       </c>
       <c r="R36" s="20" t="n">
-        <v>0.00387356</v>
+        <v>0.0039</v>
       </c>
       <c r="S36" s="20" t="n">
-        <v>0.00387356</v>
+        <v>0.0039</v>
       </c>
       <c r="T36" s="20" t="n">
-        <v>0.00387356</v>
+        <v>0.0039</v>
       </c>
       <c r="U36" s="20" t="n">
-        <v>0.00387356</v>
+        <v>0.0039</v>
       </c>
       <c r="V36" s="11" t="n"/>
       <c r="W36" s="19" t="n"/>
@@ -1935,31 +1935,31 @@
       </c>
       <c r="L37" s="11" t="n"/>
       <c r="M37" s="20" t="n">
-        <v>0.00185933</v>
+        <v>0.0019</v>
       </c>
       <c r="N37" s="20" t="n">
-        <v>0.00185933</v>
+        <v>0.0019</v>
       </c>
       <c r="O37" s="20" t="n">
-        <v>0.00185933</v>
+        <v>0.0019</v>
       </c>
       <c r="P37" s="20" t="n">
-        <v>0.00185933</v>
+        <v>0.0019</v>
       </c>
       <c r="Q37" s="20" t="n">
-        <v>0.00185933</v>
+        <v>0.0019</v>
       </c>
       <c r="R37" s="20" t="n">
-        <v>0.00185933</v>
+        <v>0.0019</v>
       </c>
       <c r="S37" s="20" t="n">
-        <v>0.00185933</v>
+        <v>0.0019</v>
       </c>
       <c r="T37" s="20" t="n">
-        <v>0.00185933</v>
+        <v>0.0019</v>
       </c>
       <c r="U37" s="20" t="n">
-        <v>0.00185933</v>
+        <v>0.0019</v>
       </c>
       <c r="V37" s="11" t="n"/>
       <c r="W37" s="19" t="n"/>
@@ -1995,31 +1995,31 @@
       </c>
       <c r="L38" s="11" t="n"/>
       <c r="M38" s="20" t="n">
-        <v>0.01053611</v>
+        <v>0.0105</v>
       </c>
       <c r="N38" s="20" t="n">
-        <v>0.01053611</v>
+        <v>0.0105</v>
       </c>
       <c r="O38" s="20" t="n">
-        <v>0.01053611</v>
+        <v>0.0105</v>
       </c>
       <c r="P38" s="20" t="n">
-        <v>0.01053611</v>
+        <v>0.0105</v>
       </c>
       <c r="Q38" s="20" t="n">
-        <v>0.01053611</v>
+        <v>0.0105</v>
       </c>
       <c r="R38" s="20" t="n">
-        <v>0.01053611</v>
+        <v>0.0105</v>
       </c>
       <c r="S38" s="20" t="n">
-        <v>0.01053611</v>
+        <v>0.0105</v>
       </c>
       <c r="T38" s="20" t="n">
-        <v>0.01053611</v>
+        <v>0.0105</v>
       </c>
       <c r="U38" s="20" t="n">
-        <v>0.01053611</v>
+        <v>0.0105</v>
       </c>
       <c r="V38" s="11" t="n"/>
       <c r="W38" s="19" t="n"/>
@@ -2055,31 +2055,31 @@
       </c>
       <c r="L39" s="11" t="n"/>
       <c r="M39" s="20" t="n">
-        <v>0.005423</v>
+        <v>0.0054</v>
       </c>
       <c r="N39" s="20" t="n">
-        <v>0.005423</v>
+        <v>0.0054</v>
       </c>
       <c r="O39" s="20" t="n">
-        <v>0.005423</v>
+        <v>0.0054</v>
       </c>
       <c r="P39" s="20" t="n">
-        <v>0.005423</v>
+        <v>0.0054</v>
       </c>
       <c r="Q39" s="20" t="n">
-        <v>0.005423</v>
+        <v>0.0054</v>
       </c>
       <c r="R39" s="20" t="n">
-        <v>0.005423</v>
+        <v>0.0054</v>
       </c>
       <c r="S39" s="20" t="n">
-        <v>0.005423</v>
+        <v>0.0054</v>
       </c>
       <c r="T39" s="20" t="n">
-        <v>0.005423</v>
+        <v>0.0054</v>
       </c>
       <c r="U39" s="20" t="n">
-        <v>0.005423</v>
+        <v>0.0054</v>
       </c>
       <c r="V39" s="11" t="n"/>
       <c r="W39" s="19" t="n"/>
@@ -2171,31 +2171,31 @@
       </c>
       <c r="L42" s="11" t="n"/>
       <c r="M42" s="20" t="n">
-        <v>0.02479078</v>
+        <v>0.0248</v>
       </c>
       <c r="N42" s="20" t="n">
-        <v>0.02479078</v>
+        <v>0.0248</v>
       </c>
       <c r="O42" s="20" t="n">
-        <v>0.02479078</v>
+        <v>0.0248</v>
       </c>
       <c r="P42" s="20" t="n">
-        <v>0.02479078</v>
+        <v>0.0248</v>
       </c>
       <c r="Q42" s="20" t="n">
-        <v>0.02479078</v>
+        <v>0.0248</v>
       </c>
       <c r="R42" s="20" t="n">
-        <v>0.02479078</v>
+        <v>0.0248</v>
       </c>
       <c r="S42" s="20" t="n">
-        <v>0.02479078</v>
+        <v>0.0248</v>
       </c>
       <c r="T42" s="20" t="n">
-        <v>0.02479078</v>
+        <v>0.0248</v>
       </c>
       <c r="U42" s="20" t="n">
-        <v>0.02479078</v>
+        <v>0.0248</v>
       </c>
       <c r="V42" s="11" t="n"/>
       <c r="W42" s="19" t="n"/>
@@ -2287,31 +2287,31 @@
       </c>
       <c r="L45" s="11" t="n"/>
       <c r="M45" s="20" t="n">
-        <v>0.04648278</v>
+        <v>0.0465</v>
       </c>
       <c r="N45" s="20" t="n">
-        <v>0.04648278</v>
+        <v>0.0465</v>
       </c>
       <c r="O45" s="20" t="n">
-        <v>0.04648278</v>
+        <v>0.0465</v>
       </c>
       <c r="P45" s="20" t="n">
-        <v>0.04648278</v>
+        <v>0.0465</v>
       </c>
       <c r="Q45" s="20" t="n">
-        <v>0.04648278</v>
+        <v>0.0465</v>
       </c>
       <c r="R45" s="20" t="n">
-        <v>0.04648278</v>
+        <v>0.0465</v>
       </c>
       <c r="S45" s="20" t="n">
-        <v>0.04648278</v>
+        <v>0.0465</v>
       </c>
       <c r="T45" s="20" t="n">
-        <v>0.04648278</v>
+        <v>0.0465</v>
       </c>
       <c r="U45" s="20" t="n">
-        <v>0.04648278</v>
+        <v>0.0465</v>
       </c>
       <c r="V45" s="11" t="n"/>
       <c r="W45" s="19" t="n"/>
@@ -2403,7 +2403,7 @@
       </c>
       <c r="L48" s="11" t="n"/>
       <c r="M48" s="20" t="n">
-        <v>0.023706</v>
+        <v>0.0237</v>
       </c>
       <c r="N48" s="17" t="n"/>
       <c r="O48" s="17" t="n"/>
@@ -2447,7 +2447,7 @@
       </c>
       <c r="L49" s="11" t="n"/>
       <c r="M49" s="20" t="n">
-        <v>0.023706</v>
+        <v>0.0237</v>
       </c>
       <c r="N49" s="17" t="n"/>
       <c r="O49" s="17" t="n"/>
@@ -2547,10 +2547,10 @@
       </c>
       <c r="L52" s="11" t="n"/>
       <c r="M52" s="20" t="n">
-        <v>0.159058</v>
+        <v>0.1591</v>
       </c>
       <c r="N52" s="20" t="n">
-        <v>0.159058</v>
+        <v>0.1591</v>
       </c>
       <c r="O52" s="17" t="n"/>
       <c r="P52" s="17" t="n"/>
@@ -2589,22 +2589,22 @@
         <v>52997594.52</v>
       </c>
       <c r="K53" s="17" t="n">
-        <v>14.780848</v>
+        <v>14.780847</v>
       </c>
       <c r="L53" s="11" t="n"/>
       <c r="M53" s="17" t="n"/>
       <c r="N53" s="17" t="n"/>
       <c r="O53" s="20" t="n">
-        <v>3.695212</v>
+        <v>3.6952</v>
       </c>
       <c r="P53" s="20" t="n">
-        <v>3.695212</v>
+        <v>3.6952</v>
       </c>
       <c r="Q53" s="20" t="n">
-        <v>3.695212</v>
+        <v>3.6952</v>
       </c>
       <c r="R53" s="20" t="n">
-        <v>3.695212</v>
+        <v>3.6952</v>
       </c>
       <c r="S53" s="17" t="n"/>
       <c r="T53" s="17" t="n"/>
@@ -2645,16 +2645,16 @@
       <c r="M54" s="17" t="n"/>
       <c r="N54" s="17" t="n"/>
       <c r="O54" s="20" t="n">
-        <v>0.18715525</v>
+        <v>0.1872</v>
       </c>
       <c r="P54" s="20" t="n">
-        <v>0.18715525</v>
+        <v>0.1872</v>
       </c>
       <c r="Q54" s="20" t="n">
-        <v>0.18715525</v>
+        <v>0.1872</v>
       </c>
       <c r="R54" s="20" t="n">
-        <v>0.18715525</v>
+        <v>0.1872</v>
       </c>
       <c r="S54" s="17" t="n"/>
       <c r="T54" s="17" t="n"/>
@@ -2694,16 +2694,16 @@
       <c r="L55" s="11" t="n"/>
       <c r="M55" s="17" t="n"/>
       <c r="N55" s="20" t="n">
-        <v>0.652855</v>
+        <v>0.6529</v>
       </c>
       <c r="O55" s="20" t="n">
-        <v>0.652855</v>
+        <v>0.6529</v>
       </c>
       <c r="P55" s="20" t="n">
-        <v>0.652855</v>
+        <v>0.6529</v>
       </c>
       <c r="Q55" s="20" t="n">
-        <v>0.652855</v>
+        <v>0.6529</v>
       </c>
       <c r="R55" s="17" t="n"/>
       <c r="S55" s="17" t="n"/>
@@ -2739,14 +2739,14 @@
         <v>5398824</v>
       </c>
       <c r="K56" s="17" t="n">
-        <v>1.505714</v>
+        <v>1.505713</v>
       </c>
       <c r="L56" s="11" t="n"/>
       <c r="M56" s="20" t="n">
-        <v>0.752857</v>
+        <v>0.7529</v>
       </c>
       <c r="N56" s="20" t="n">
-        <v>0.752857</v>
+        <v>0.7529</v>
       </c>
       <c r="O56" s="17" t="n"/>
       <c r="P56" s="17" t="n"/>
@@ -2793,16 +2793,16 @@
       <c r="O57" s="17" t="n"/>
       <c r="P57" s="17" t="n"/>
       <c r="Q57" s="20" t="n">
-        <v>0.55906525</v>
+        <v>0.5591</v>
       </c>
       <c r="R57" s="20" t="n">
-        <v>0.55906525</v>
+        <v>0.5591</v>
       </c>
       <c r="S57" s="20" t="n">
-        <v>0.55906525</v>
+        <v>0.5591</v>
       </c>
       <c r="T57" s="20" t="n">
-        <v>0.55906525</v>
+        <v>0.5591</v>
       </c>
       <c r="U57" s="17" t="n"/>
       <c r="V57" s="11" t="n"/>
@@ -2843,16 +2843,16 @@
       <c r="O58" s="17" t="n"/>
       <c r="P58" s="17" t="n"/>
       <c r="Q58" s="20" t="n">
-        <v>0.013324</v>
+        <v>0.0133</v>
       </c>
       <c r="R58" s="20" t="n">
-        <v>0.013324</v>
+        <v>0.0133</v>
       </c>
       <c r="S58" s="20" t="n">
-        <v>0.013324</v>
+        <v>0.0133</v>
       </c>
       <c r="T58" s="20" t="n">
-        <v>0.013324</v>
+        <v>0.0133</v>
       </c>
       <c r="U58" s="17" t="n"/>
       <c r="V58" s="11" t="n"/>
@@ -2945,10 +2945,10 @@
       </c>
       <c r="L61" s="11" t="n"/>
       <c r="M61" s="20" t="n">
-        <v>0.110314</v>
+        <v>0.1103</v>
       </c>
       <c r="N61" s="20" t="n">
-        <v>0.110314</v>
+        <v>0.1103</v>
       </c>
       <c r="O61" s="17" t="n"/>
       <c r="P61" s="17" t="n"/>
@@ -2993,16 +2993,16 @@
       <c r="M62" s="17" t="n"/>
       <c r="N62" s="17" t="n"/>
       <c r="O62" s="20" t="n">
-        <v>1.70853283</v>
+        <v>1.7085</v>
       </c>
       <c r="P62" s="20" t="n">
-        <v>3.41706567</v>
+        <v>3.4171</v>
       </c>
       <c r="Q62" s="20" t="n">
-        <v>3.41706567</v>
+        <v>3.4171</v>
       </c>
       <c r="R62" s="20" t="n">
-        <v>1.70853283</v>
+        <v>1.7085</v>
       </c>
       <c r="S62" s="17" t="n"/>
       <c r="T62" s="17" t="n"/>
@@ -3043,16 +3043,16 @@
       <c r="M63" s="17" t="n"/>
       <c r="N63" s="17" t="n"/>
       <c r="O63" s="20" t="n">
-        <v>0.12746625</v>
+        <v>0.1275</v>
       </c>
       <c r="P63" s="20" t="n">
-        <v>0.12746625</v>
+        <v>0.1275</v>
       </c>
       <c r="Q63" s="20" t="n">
-        <v>0.12746625</v>
+        <v>0.1275</v>
       </c>
       <c r="R63" s="20" t="n">
-        <v>0.12746625</v>
+        <v>0.1275</v>
       </c>
       <c r="S63" s="17" t="n"/>
       <c r="T63" s="17" t="n"/>
@@ -3092,16 +3092,16 @@
       <c r="L64" s="11" t="n"/>
       <c r="M64" s="17" t="n"/>
       <c r="N64" s="20" t="n">
-        <v>0.5159792</v>
+        <v>0.516</v>
       </c>
       <c r="O64" s="20" t="n">
-        <v>0.5159792</v>
+        <v>0.516</v>
       </c>
       <c r="P64" s="20" t="n">
-        <v>0.5159792</v>
+        <v>0.516</v>
       </c>
       <c r="Q64" s="20" t="n">
-        <v>0.1300014</v>
+        <v>0.13</v>
       </c>
       <c r="R64" s="17" t="n"/>
       <c r="S64" s="17" t="n"/>
@@ -3141,10 +3141,10 @@
       </c>
       <c r="L65" s="11" t="n"/>
       <c r="M65" s="20" t="n">
-        <v>0.55015167</v>
+        <v>0.5502</v>
       </c>
       <c r="N65" s="20" t="n">
-        <v>0.45365733</v>
+        <v>0.4537</v>
       </c>
       <c r="O65" s="17" t="n"/>
       <c r="P65" s="17" t="n"/>
@@ -3183,7 +3183,7 @@
         <v>5345496</v>
       </c>
       <c r="K66" s="17" t="n">
-        <v>1.490841</v>
+        <v>1.49084</v>
       </c>
       <c r="L66" s="11" t="n"/>
       <c r="M66" s="17" t="n"/>
@@ -3191,16 +3191,16 @@
       <c r="O66" s="17" t="n"/>
       <c r="P66" s="17" t="n"/>
       <c r="Q66" s="20" t="n">
-        <v>0.37271025</v>
+        <v>0.3727</v>
       </c>
       <c r="R66" s="20" t="n">
-        <v>0.37271025</v>
+        <v>0.3727</v>
       </c>
       <c r="S66" s="20" t="n">
-        <v>0.37271025</v>
+        <v>0.3727</v>
       </c>
       <c r="T66" s="20" t="n">
-        <v>0.37271025</v>
+        <v>0.3727</v>
       </c>
       <c r="U66" s="17" t="n"/>
       <c r="V66" s="11" t="n"/>
@@ -3241,16 +3241,16 @@
       <c r="O67" s="17" t="n"/>
       <c r="P67" s="17" t="n"/>
       <c r="Q67" s="20" t="n">
-        <v>0.00888275</v>
+        <v>0.0089</v>
       </c>
       <c r="R67" s="20" t="n">
-        <v>0.00888275</v>
+        <v>0.0089</v>
       </c>
       <c r="S67" s="20" t="n">
-        <v>0.00888275</v>
+        <v>0.0089</v>
       </c>
       <c r="T67" s="20" t="n">
-        <v>0.00888275</v>
+        <v>0.0089</v>
       </c>
       <c r="U67" s="17" t="n"/>
       <c r="V67" s="11" t="n"/>
@@ -3426,10 +3426,10 @@
       <c r="R72" s="17" t="n"/>
       <c r="S72" s="17" t="n"/>
       <c r="T72" s="20" t="n">
-        <v>0.238524</v>
+        <v>0.2385</v>
       </c>
       <c r="U72" s="20" t="n">
-        <v>0.119262</v>
+        <v>0.1193</v>
       </c>
       <c r="V72" s="11" t="n"/>
       <c r="W72" s="19" t="n"/>
@@ -3472,10 +3472,10 @@
       <c r="R73" s="17" t="n"/>
       <c r="S73" s="17" t="n"/>
       <c r="T73" s="20" t="n">
-        <v>0.06340867</v>
+        <v>0.0634</v>
       </c>
       <c r="U73" s="20" t="n">
-        <v>0.03170433</v>
+        <v>0.0317</v>
       </c>
       <c r="V73" s="11" t="n"/>
       <c r="W73" s="19" t="n"/>
@@ -3518,10 +3518,10 @@
       <c r="R74" s="17" t="n"/>
       <c r="S74" s="17" t="n"/>
       <c r="T74" s="20" t="n">
-        <v>0.022808</v>
+        <v>0.0228</v>
       </c>
       <c r="U74" s="20" t="n">
-        <v>0.011404</v>
+        <v>0.0114</v>
       </c>
       <c r="V74" s="11" t="n"/>
       <c r="W74" s="19" t="n"/>
@@ -3564,10 +3564,10 @@
       <c r="R75" s="17" t="n"/>
       <c r="S75" s="17" t="n"/>
       <c r="T75" s="20" t="n">
-        <v>0.16730133</v>
+        <v>0.1673</v>
       </c>
       <c r="U75" s="20" t="n">
-        <v>0.08365067</v>
+        <v>0.0837</v>
       </c>
       <c r="V75" s="11" t="n"/>
       <c r="W75" s="19" t="n"/>
@@ -3610,10 +3610,10 @@
       <c r="R76" s="17" t="n"/>
       <c r="S76" s="17" t="n"/>
       <c r="T76" s="20" t="n">
-        <v>0.02368733</v>
+        <v>0.0237</v>
       </c>
       <c r="U76" s="20" t="n">
-        <v>0.01184367</v>
+        <v>0.0118</v>
       </c>
       <c r="V76" s="11" t="n"/>
       <c r="W76" s="19" t="n"/>
@@ -3705,7 +3705,7 @@
       </c>
       <c r="L79" s="11" t="n"/>
       <c r="M79" s="20" t="n">
-        <v>0.315455</v>
+        <v>0.3155</v>
       </c>
       <c r="N79" s="17" t="n"/>
       <c r="O79" s="17" t="n"/>
@@ -3736,20 +3736,20 @@
         </is>
       </c>
       <c r="H80" s="17" t="n">
-        <v>135.74925</v>
+        <v>135.7493</v>
       </c>
       <c r="I80" s="18" t="n">
         <v>5500</v>
       </c>
       <c r="J80" s="18" t="n">
-        <v>746620.8749999999</v>
+        <v>746621.15</v>
       </c>
       <c r="K80" s="17" t="n">
         <v>0.20823</v>
       </c>
       <c r="L80" s="11" t="n"/>
       <c r="M80" s="20" t="n">
-        <v>0.20823</v>
+        <v>0.2082</v>
       </c>
       <c r="N80" s="17" t="n"/>
       <c r="O80" s="17" t="n"/>
@@ -3780,27 +3780,27 @@
         </is>
       </c>
       <c r="H81" s="17" t="n">
-        <v>135.74925</v>
+        <v>135.7493</v>
       </c>
       <c r="I81" s="18" t="n">
         <v>255550</v>
       </c>
       <c r="J81" s="18" t="n">
-        <v>34690720.8375</v>
+        <v>34690733.615</v>
       </c>
       <c r="K81" s="17" t="n">
-        <v>9.675122999999999</v>
+        <v>9.675126000000001</v>
       </c>
       <c r="L81" s="11" t="n"/>
       <c r="M81" s="17" t="n"/>
       <c r="N81" s="20" t="n">
-        <v>1.20939038</v>
+        <v>1.2094</v>
       </c>
       <c r="O81" s="20" t="n">
-        <v>4.78931444</v>
+        <v>4.7893</v>
       </c>
       <c r="P81" s="20" t="n">
-        <v>3.67641818</v>
+        <v>3.6764</v>
       </c>
       <c r="Q81" s="17" t="n"/>
       <c r="R81" s="17" t="n"/>
@@ -3842,10 +3842,10 @@
       <c r="L82" s="11" t="n"/>
       <c r="M82" s="17" t="n"/>
       <c r="N82" s="20" t="n">
-        <v>0.2472935</v>
+        <v>0.2473</v>
       </c>
       <c r="O82" s="20" t="n">
-        <v>0.2472935</v>
+        <v>0.2473</v>
       </c>
       <c r="P82" s="17" t="n"/>
       <c r="Q82" s="17" t="n"/>
@@ -3891,13 +3891,13 @@
       <c r="O83" s="17" t="n"/>
       <c r="P83" s="17" t="n"/>
       <c r="Q83" s="20" t="n">
-        <v>0.1845066</v>
+        <v>0.1845</v>
       </c>
       <c r="R83" s="20" t="n">
-        <v>0.34594988</v>
+        <v>0.3459</v>
       </c>
       <c r="S83" s="20" t="n">
-        <v>2.23714252</v>
+        <v>2.2371</v>
       </c>
       <c r="T83" s="17" t="n"/>
       <c r="U83" s="17" t="n"/>
@@ -3936,10 +3936,10 @@
       <c r="L84" s="11" t="n"/>
       <c r="M84" s="17" t="n"/>
       <c r="N84" s="20" t="n">
-        <v>0.5019045</v>
+        <v>0.5019</v>
       </c>
       <c r="O84" s="20" t="n">
-        <v>0.5019045</v>
+        <v>0.5019</v>
       </c>
       <c r="P84" s="17" t="n"/>
       <c r="Q84" s="17" t="n"/>
@@ -3977,7 +3977,7 @@
         <v>5345496</v>
       </c>
       <c r="K85" s="17" t="n">
-        <v>1.490841</v>
+        <v>1.49084</v>
       </c>
       <c r="L85" s="11" t="n"/>
       <c r="M85" s="17" t="n"/>
@@ -3988,10 +3988,10 @@
       <c r="R85" s="17" t="n"/>
       <c r="S85" s="17" t="n"/>
       <c r="T85" s="20" t="n">
-        <v>0.7454205</v>
+        <v>0.7454</v>
       </c>
       <c r="U85" s="20" t="n">
-        <v>0.7454205</v>
+        <v>0.7454</v>
       </c>
       <c r="V85" s="11" t="n"/>
       <c r="W85" s="19" t="n"/>
@@ -4034,10 +4034,10 @@
       <c r="R86" s="17" t="n"/>
       <c r="S86" s="17" t="n"/>
       <c r="T86" s="20" t="n">
-        <v>0.0177655</v>
+        <v>0.0178</v>
       </c>
       <c r="U86" s="20" t="n">
-        <v>0.0177655</v>
+        <v>0.017</v>
       </c>
       <c r="V86" s="11" t="n"/>
       <c r="W86" s="19" t="n"/>
@@ -4162,7 +4162,7 @@
       <c r="L90" s="11" t="n"/>
       <c r="M90" s="17" t="n"/>
       <c r="N90" s="20" t="n">
-        <v>0.63532</v>
+        <v>0.6353</v>
       </c>
       <c r="O90" s="17" t="n"/>
       <c r="P90" s="17" t="n"/>
@@ -4201,25 +4201,25 @@
         <v>61584381.18</v>
       </c>
       <c r="K91" s="17" t="n">
-        <v>17.175673</v>
+        <v>17.175672</v>
       </c>
       <c r="L91" s="11" t="n"/>
       <c r="M91" s="17" t="n"/>
       <c r="N91" s="17" t="n"/>
       <c r="O91" s="20" t="n">
-        <v>0.95420406</v>
+        <v>0.9542</v>
       </c>
       <c r="P91" s="20" t="n">
-        <v>5.18136414</v>
+        <v>5.1814</v>
       </c>
       <c r="Q91" s="20" t="n">
-        <v>4.29391825</v>
+        <v>4.2939</v>
       </c>
       <c r="R91" s="20" t="n">
-        <v>3.37309328</v>
+        <v>3.3731</v>
       </c>
       <c r="S91" s="20" t="n">
-        <v>3.37309328</v>
+        <v>3.3731</v>
       </c>
       <c r="T91" s="17" t="n"/>
       <c r="U91" s="17" t="n"/>
@@ -4259,19 +4259,19 @@
       <c r="M92" s="17" t="n"/>
       <c r="N92" s="17" t="n"/>
       <c r="O92" s="20" t="n">
-        <v>0.74386839</v>
+        <v>0.7439</v>
       </c>
       <c r="P92" s="20" t="n">
-        <v>9.231605220000001</v>
+        <v>9.2316</v>
       </c>
       <c r="Q92" s="20" t="n">
-        <v>3.34740775</v>
+        <v>3.3474</v>
       </c>
       <c r="R92" s="20" t="n">
-        <v>0.03337482</v>
+        <v>0.0334</v>
       </c>
       <c r="S92" s="20" t="n">
-        <v>0.03337482</v>
+        <v>0.0334</v>
       </c>
       <c r="T92" s="17" t="n"/>
       <c r="U92" s="17" t="n"/>
@@ -4311,19 +4311,19 @@
       <c r="M93" s="17" t="n"/>
       <c r="N93" s="17" t="n"/>
       <c r="O93" s="20" t="n">
-        <v>0.15502667</v>
+        <v>0.155</v>
       </c>
       <c r="P93" s="20" t="n">
-        <v>0.31005333</v>
+        <v>0.3101</v>
       </c>
       <c r="Q93" s="20" t="n">
-        <v>0.23254</v>
+        <v>0.2325</v>
       </c>
       <c r="R93" s="20" t="n">
-        <v>0.11627</v>
+        <v>0.1163</v>
       </c>
       <c r="S93" s="20" t="n">
-        <v>0.11627</v>
+        <v>0.1163</v>
       </c>
       <c r="T93" s="17" t="n"/>
       <c r="U93" s="17" t="n"/>
@@ -4363,19 +4363,19 @@
       <c r="M94" s="17" t="n"/>
       <c r="N94" s="17" t="n"/>
       <c r="O94" s="20" t="n">
-        <v>0.39988625</v>
+        <v>0.3999</v>
       </c>
       <c r="P94" s="20" t="n">
-        <v>0.39988625</v>
+        <v>0.3999</v>
       </c>
       <c r="Q94" s="20" t="n">
-        <v>0.39988625</v>
+        <v>0.3999</v>
       </c>
       <c r="R94" s="20" t="n">
-        <v>0.19994313</v>
+        <v>0.1999</v>
       </c>
       <c r="S94" s="20" t="n">
-        <v>0.19994313</v>
+        <v>0.1999</v>
       </c>
       <c r="T94" s="17" t="n"/>
       <c r="U94" s="17" t="n"/>
@@ -4414,13 +4414,13 @@
       <c r="L95" s="11" t="n"/>
       <c r="M95" s="17" t="n"/>
       <c r="N95" s="20" t="n">
-        <v>1.22339225</v>
+        <v>1.2234</v>
       </c>
       <c r="O95" s="20" t="n">
-        <v>1.63118967</v>
+        <v>1.6312</v>
       </c>
       <c r="P95" s="20" t="n">
-        <v>2.03898708</v>
+        <v>2.039</v>
       </c>
       <c r="Q95" s="17" t="n"/>
       <c r="R95" s="17" t="n"/>
@@ -4467,10 +4467,10 @@
       <c r="Q96" s="17" t="n"/>
       <c r="R96" s="17" t="n"/>
       <c r="S96" s="20" t="n">
-        <v>0.6817879999999999</v>
+        <v>0.6818</v>
       </c>
       <c r="T96" s="20" t="n">
-        <v>0.340894</v>
+        <v>0.3409</v>
       </c>
       <c r="U96" s="17" t="n"/>
       <c r="V96" s="11" t="n"/>
@@ -4503,7 +4503,7 @@
         <v>16036488</v>
       </c>
       <c r="K97" s="17" t="n">
-        <v>4.472522</v>
+        <v>4.472521</v>
       </c>
       <c r="L97" s="11" t="n"/>
       <c r="M97" s="17" t="n"/>
@@ -4513,10 +4513,10 @@
       <c r="Q97" s="17" t="n"/>
       <c r="R97" s="17" t="n"/>
       <c r="S97" s="20" t="n">
-        <v>2.98168133</v>
+        <v>2.9817</v>
       </c>
       <c r="T97" s="20" t="n">
-        <v>1.49084067</v>
+        <v>1.4908</v>
       </c>
       <c r="U97" s="17" t="n"/>
       <c r="V97" s="11" t="n"/>
@@ -4559,10 +4559,10 @@
       <c r="Q98" s="17" t="n"/>
       <c r="R98" s="17" t="n"/>
       <c r="S98" s="20" t="n">
-        <v>0.04737467</v>
+        <v>0.0474</v>
       </c>
       <c r="T98" s="20" t="n">
-        <v>0.02368733</v>
+        <v>0.0237</v>
       </c>
       <c r="U98" s="17" t="n"/>
       <c r="V98" s="11" t="n"/>
@@ -4605,10 +4605,10 @@
       <c r="Q99" s="17" t="n"/>
       <c r="R99" s="17" t="n"/>
       <c r="S99" s="20" t="n">
-        <v>0.017388</v>
+        <v>0.017</v>
       </c>
       <c r="T99" s="20" t="n">
-        <v>0.008694</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="U99" s="17" t="n"/>
       <c r="V99" s="11" t="n"/>
@@ -4783,7 +4783,7 @@
       <c r="K106" s="33" t="n"/>
       <c r="L106" s="28" t="n"/>
       <c r="M106" s="34" t="n">
-        <v>2.312</v>
+        <v>2.313</v>
       </c>
       <c r="N106" s="34" t="n">
         <v>6.631</v>
@@ -4807,7 +4807,7 @@
         <v>4.274</v>
       </c>
       <c r="U106" s="34" t="n">
-        <v>1.19</v>
+        <v>1.189</v>
       </c>
       <c r="V106" s="28" t="n"/>
       <c r="W106" s="29" t="n"/>
@@ -4829,28 +4829,28 @@
       <c r="K107" s="33" t="n"/>
       <c r="L107" s="28" t="n"/>
       <c r="M107" s="34" t="n">
-        <v>2.312</v>
+        <v>2.313</v>
       </c>
       <c r="N107" s="34" t="n">
-        <v>8.943</v>
+        <v>8.944000000000001</v>
       </c>
       <c r="O107" s="34" t="n">
         <v>25.422</v>
       </c>
       <c r="P107" s="34" t="n">
-        <v>55.025</v>
+        <v>55.026</v>
       </c>
       <c r="Q107" s="34" t="n">
-        <v>72.816</v>
+        <v>72.81699999999999</v>
       </c>
       <c r="R107" s="34" t="n">
-        <v>83.726</v>
+        <v>83.727</v>
       </c>
       <c r="S107" s="34" t="n">
         <v>94.53700000000001</v>
       </c>
       <c r="T107" s="34" t="n">
-        <v>98.81</v>
+        <v>98.81100000000001</v>
       </c>
       <c r="U107" s="34" t="n">
         <v>100</v>
@@ -4975,28 +4975,28 @@
       <c r="K110" s="33" t="n"/>
       <c r="L110" s="37" t="n"/>
       <c r="M110" s="34" t="n">
-        <v>-2.312</v>
+        <v>-2.313</v>
       </c>
       <c r="N110" s="34" t="n">
-        <v>-8.943</v>
+        <v>-8.944000000000001</v>
       </c>
       <c r="O110" s="34" t="n">
         <v>-25.422</v>
       </c>
       <c r="P110" s="34" t="n">
-        <v>-55.025</v>
+        <v>-55.026</v>
       </c>
       <c r="Q110" s="34" t="n">
-        <v>-72.816</v>
+        <v>-72.81699999999999</v>
       </c>
       <c r="R110" s="34" t="n">
-        <v>-83.726</v>
+        <v>-83.727</v>
       </c>
       <c r="S110" s="34" t="n">
         <v>-94.53700000000001</v>
       </c>
       <c r="T110" s="34" t="n">
-        <v>-98.81</v>
+        <v>-98.81100000000001</v>
       </c>
       <c r="U110" s="34" t="n">
         <v>-100</v>
@@ -5294,7 +5294,7 @@
         </is>
       </c>
       <c r="B2" s="46" t="n">
-        <v>2.312</v>
+        <v>2.313</v>
       </c>
       <c r="C2" s="46" t="n">
         <v>0</v>
@@ -5310,7 +5310,7 @@
         </is>
       </c>
       <c r="B3" s="46" t="n">
-        <v>8.943</v>
+        <v>8.944000000000001</v>
       </c>
       <c r="C3" s="46" t="n">
         <v>0</v>
@@ -5342,7 +5342,7 @@
         </is>
       </c>
       <c r="B5" s="46" t="n">
-        <v>55.025</v>
+        <v>55.026</v>
       </c>
       <c r="C5" s="46" t="n">
         <v>0</v>
@@ -5358,7 +5358,7 @@
         </is>
       </c>
       <c r="B6" s="46" t="n">
-        <v>72.816</v>
+        <v>72.81699999999999</v>
       </c>
       <c r="C6" s="46" t="n">
         <v>0</v>
@@ -5371,7 +5371,7 @@
         </is>
       </c>
       <c r="B7" s="46" t="n">
-        <v>83.726</v>
+        <v>83.727</v>
       </c>
       <c r="C7" s="46" t="n">
         <v>0</v>
@@ -5397,7 +5397,7 @@
         </is>
       </c>
       <c r="B9" s="46" t="n">
-        <v>98.81</v>
+        <v>98.81100000000001</v>
       </c>
       <c r="C9" s="46" t="n">
         <v>0</v>

</xml_diff>